<commit_message>
R04 and R10: measured where it matters, severity by size and persistence
R04 fired on almost every real company: 1% of revenue in other income is a bar
nearly every group passes, and it was always High.
- R04 now measures other income against EBITDA, the base of the price: it fires
  above 10% and is High above 25% (Toyota 52%: High; EDP 17%, Amorim 11%,
  Duriva 22%: Medium; Velmora 4.5%: no finding)
- R10 still fires on any year below 70%, but is High only when the years
  analysed together convert less than 70%: one weak year is often working
  capital timing (EDP FY25 67%, period 81%: Medium; Toyota 39%, Amorim 44%,
  Duriva 67%: High)
- graded severity is a rule field shown with the threshold; the Excel template
  (Duriva and Velmora) carries the same metrics and formulas, recalculated by
  Excel, so the parity test still holds

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/DD_template_velmora.xlsx
+++ b/data/DD_template_velmora.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yesdo\Documents\projetos\dd-assistant\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F094B1-1F2D-4875-A768-689940D9778A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09D84EE-33AF-40B9-864D-024EC0653B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Leia-me" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="446">
   <si>
     <t>Due Diligence Assistant — template de análise (módulo 1)</t>
   </si>
@@ -1366,6 +1366,18 @@
   </si>
   <si>
     <t>Empresa desenhada sem problemas plantados, para medir alarmes falsos. Foi criada por quem conhece as regras: zero alertas é um teste de sanidade, não uma medida independente.</t>
+  </si>
+  <si>
+    <t>Outros rendimentos (% do EBITDA)</t>
+  </si>
+  <si>
+    <t>Outros rendimentos / EBITDA reportado</t>
+  </si>
+  <si>
+    <t>Conversão de caixa acumulada (anos analisados)</t>
+  </si>
+  <si>
+    <t>Soma da caixa gerada pelas operações / soma do EBITDA, até ao ano</t>
   </si>
 </sst>
 </file>
@@ -1914,23 +1926,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="17.600000000000001" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>440</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
@@ -1938,7 +1950,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1946,7 +1958,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
@@ -1954,7 +1966,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
@@ -1962,7 +1974,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:2" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
@@ -1970,7 +1982,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -1978,7 +1990,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>13</v>
       </c>
@@ -1998,7 +2010,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N25"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -2013,17 +2025,17 @@
     <col min="12" max="12" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="17.600000000000001" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:14" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="15.45" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E3" s="5" t="str">
         <f>"Alertas: "&amp;$N$3&amp;"   ·   Alta: "&amp;COUNTIFS(Regras!M5:M24,"Sim",Regras!O5:O24,"Alta")&amp;"   ·   Média: "&amp;COUNTIFS(Regras!M5:M24,"Sim",Regras!O5:O24,"Média")&amp;"   ·   Baixa: "&amp;COUNTIFS(Regras!M5:M24,"Sim",Regras!O5:O24,"Baixa")&amp;"   ·   Por rever: "&amp;($N$3-COUNTIF(K6:K25,"Aceite")-COUNTIF(K6:K25,"Descartado"))</f>
         <v>Alertas: 0   ·   Alta: 0   ·   Média: 0   ·   Baixa: 0   ·   Por rever: 0</v>
@@ -2033,7 +2045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="24.9" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>16</v>
       </c>
@@ -2071,7 +2083,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="str">
         <f>IF(1&lt;=$N$3,1,"")</f>
         <v/>
@@ -2115,7 +2127,7 @@
       <c r="K6" s="11"/>
       <c r="L6" s="11"/>
     </row>
-    <row r="7" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="str">
         <f>IF(2&lt;=$N$3,2,"")</f>
         <v/>
@@ -2159,7 +2171,7 @@
       <c r="K7" s="11"/>
       <c r="L7" s="11"/>
     </row>
-    <row r="8" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="str">
         <f>IF(3&lt;=$N$3,3,"")</f>
         <v/>
@@ -2203,7 +2215,7 @@
       <c r="K8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="str">
         <f>IF(4&lt;=$N$3,4,"")</f>
         <v/>
@@ -2247,7 +2259,7 @@
       <c r="K9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="str">
         <f>IF(5&lt;=$N$3,5,"")</f>
         <v/>
@@ -2291,7 +2303,7 @@
       <c r="K10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="str">
         <f>IF(6&lt;=$N$3,6,"")</f>
         <v/>
@@ -2335,7 +2347,7 @@
       <c r="K11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="str">
         <f>IF(7&lt;=$N$3,7,"")</f>
         <v/>
@@ -2379,7 +2391,7 @@
       <c r="K12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="str">
         <f>IF(8&lt;=$N$3,8,"")</f>
         <v/>
@@ -2423,7 +2435,7 @@
       <c r="K13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="str">
         <f>IF(9&lt;=$N$3,9,"")</f>
         <v/>
@@ -2467,7 +2479,7 @@
       <c r="K14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="str">
         <f>IF(10&lt;=$N$3,10,"")</f>
         <v/>
@@ -2511,7 +2523,7 @@
       <c r="K15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:14" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="str">
         <f>IF(11&lt;=$N$3,11,"")</f>
         <v/>
@@ -2555,7 +2567,7 @@
       <c r="K16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="str">
         <f>IF(12&lt;=$N$3,12,"")</f>
         <v/>
@@ -2599,7 +2611,7 @@
       <c r="K17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="str">
         <f>IF(13&lt;=$N$3,13,"")</f>
         <v/>
@@ -2643,7 +2655,7 @@
       <c r="K18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="str">
         <f>IF(14&lt;=$N$3,14,"")</f>
         <v/>
@@ -2687,7 +2699,7 @@
       <c r="K19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="str">
         <f>IF(15&lt;=$N$3,15,"")</f>
         <v/>
@@ -2731,7 +2743,7 @@
       <c r="K20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="str">
         <f>IF(16&lt;=$N$3,16,"")</f>
         <v/>
@@ -2775,7 +2787,7 @@
       <c r="K21" s="11"/>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="str">
         <f>IF(17&lt;=$N$3,17,"")</f>
         <v/>
@@ -2819,7 +2831,7 @@
       <c r="K22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="str">
         <f>IF(18&lt;=$N$3,18,"")</f>
         <v/>
@@ -2863,7 +2875,7 @@
       <c r="K23" s="11"/>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="str">
         <f>IF(19&lt;=$N$3,19,"")</f>
         <v/>
@@ -2907,7 +2919,7 @@
       <c r="K24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="str">
         <f>IF(20&lt;=$N$3,20,"")</f>
         <v/>
@@ -2979,24 +2991,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F86"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
     <col min="2" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.600000000000001" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>30</v>
       </c>
@@ -3016,7 +3028,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>36</v>
       </c>
@@ -3026,7 +3038,7 @@
       <c r="E5" s="13"/>
       <c r="F5" s="13"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>37</v>
       </c>
@@ -3044,7 +3056,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>39</v>
       </c>
@@ -3062,7 +3074,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>41</v>
       </c>
@@ -3080,7 +3092,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>43</v>
       </c>
@@ -3098,7 +3110,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>45</v>
       </c>
@@ -3116,7 +3128,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>47</v>
       </c>
@@ -3134,7 +3146,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>49</v>
       </c>
@@ -3152,7 +3164,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>51</v>
       </c>
@@ -3170,7 +3182,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>53</v>
       </c>
@@ -3188,7 +3200,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>55</v>
       </c>
@@ -3206,7 +3218,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>57</v>
       </c>
@@ -3224,7 +3236,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="18"/>
       <c r="B17" s="18"/>
       <c r="C17" s="18"/>
@@ -3232,7 +3244,7 @@
       <c r="E17" s="18"/>
       <c r="F17" s="18"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
         <v>59</v>
       </c>
@@ -3242,7 +3254,7 @@
       <c r="E18" s="13"/>
       <c r="F18" s="13"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>60</v>
       </c>
@@ -3262,7 +3274,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
         <v>62</v>
       </c>
@@ -3282,7 +3294,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>64</v>
       </c>
@@ -3302,7 +3314,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>66</v>
       </c>
@@ -3322,7 +3334,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>68</v>
       </c>
@@ -3342,7 +3354,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>70</v>
       </c>
@@ -3362,7 +3374,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>72</v>
       </c>
@@ -3382,7 +3394,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>74</v>
       </c>
@@ -3402,7 +3414,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
         <v>76</v>
       </c>
@@ -3422,7 +3434,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
         <v>78</v>
       </c>
@@ -3442,7 +3454,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
         <v>79</v>
       </c>
@@ -3462,7 +3474,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>81</v>
       </c>
@@ -3482,7 +3494,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
         <v>83</v>
       </c>
@@ -3502,7 +3514,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="18"/>
       <c r="B32" s="18"/>
       <c r="C32" s="18"/>
@@ -3510,7 +3522,7 @@
       <c r="E32" s="18"/>
       <c r="F32" s="18"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
         <v>85</v>
       </c>
@@ -3520,7 +3532,7 @@
       <c r="E33" s="13"/>
       <c r="F33" s="13"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
         <v>86</v>
       </c>
@@ -3538,7 +3550,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
         <v>88</v>
       </c>
@@ -3556,7 +3568,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
         <v>90</v>
       </c>
@@ -3574,7 +3586,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
         <v>92</v>
       </c>
@@ -3592,7 +3604,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
         <v>94</v>
       </c>
@@ -3610,7 +3622,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
         <v>96</v>
       </c>
@@ -3628,7 +3640,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
         <v>98</v>
       </c>
@@ -3646,7 +3658,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
         <v>100</v>
       </c>
@@ -3664,7 +3676,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
         <v>102</v>
       </c>
@@ -3682,7 +3694,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
         <v>104</v>
       </c>
@@ -3700,7 +3712,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
         <v>106</v>
       </c>
@@ -3718,7 +3730,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
         <v>108</v>
       </c>
@@ -3736,7 +3748,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
         <v>110</v>
       </c>
@@ -3754,7 +3766,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="18"/>
       <c r="B47" s="18"/>
       <c r="C47" s="18"/>
@@ -3762,7 +3774,7 @@
       <c r="E47" s="18"/>
       <c r="F47" s="18"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="12" t="s">
         <v>112</v>
       </c>
@@ -3772,7 +3784,7 @@
       <c r="E48" s="13"/>
       <c r="F48" s="13"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
         <v>113</v>
       </c>
@@ -3790,7 +3802,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="20" t="s">
         <v>115</v>
       </c>
@@ -3808,7 +3820,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="20" t="s">
         <v>117</v>
       </c>
@@ -3826,7 +3838,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="20" t="s">
         <v>119</v>
       </c>
@@ -3844,7 +3856,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="20" t="s">
         <v>121</v>
       </c>
@@ -3862,7 +3874,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="20" t="s">
         <v>123</v>
       </c>
@@ -3880,7 +3892,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="20" t="s">
         <v>125</v>
       </c>
@@ -3898,7 +3910,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="20" t="s">
         <v>127</v>
       </c>
@@ -3916,7 +3928,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="20" t="s">
         <v>129</v>
       </c>
@@ -3934,7 +3946,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="20" t="s">
         <v>433</v>
       </c>
@@ -3952,7 +3964,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="20"/>
       <c r="B59" s="15"/>
       <c r="C59" s="16"/>
@@ -3962,7 +3974,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="20"/>
       <c r="B60" s="15"/>
       <c r="C60" s="16"/>
@@ -3972,7 +3984,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="19" t="s">
         <v>133</v>
       </c>
@@ -3990,7 +4002,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="18"/>
       <c r="B62" s="18"/>
       <c r="C62" s="18"/>
@@ -3998,7 +4010,7 @@
       <c r="E62" s="18"/>
       <c r="F62" s="18"/>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="12" t="s">
         <v>135</v>
       </c>
@@ -4008,7 +4020,7 @@
       <c r="E63" s="13"/>
       <c r="F63" s="13"/>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="20" t="s">
         <v>434</v>
       </c>
@@ -4026,7 +4038,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="20" t="s">
         <v>435</v>
       </c>
@@ -4044,7 +4056,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="20" t="s">
         <v>436</v>
       </c>
@@ -4062,7 +4074,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="20"/>
       <c r="B67" s="15"/>
       <c r="C67" s="16"/>
@@ -4072,7 +4084,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="20"/>
       <c r="B68" s="15"/>
       <c r="C68" s="16"/>
@@ -4082,7 +4094,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="18"/>
       <c r="B69" s="18"/>
       <c r="C69" s="18"/>
@@ -4090,7 +4102,7 @@
       <c r="E69" s="18"/>
       <c r="F69" s="18"/>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="12" t="s">
         <v>139</v>
       </c>
@@ -4100,7 +4112,7 @@
       <c r="E70" s="13"/>
       <c r="F70" s="13"/>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="19" t="s">
         <v>140</v>
       </c>
@@ -4114,7 +4126,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="19" t="s">
         <v>141</v>
       </c>
@@ -4128,7 +4140,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="19" t="s">
         <v>142</v>
       </c>
@@ -4142,7 +4154,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="18"/>
       <c r="B74" s="18"/>
       <c r="C74" s="18"/>
@@ -4150,7 +4162,7 @@
       <c r="E74" s="18"/>
       <c r="F74" s="18"/>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="12" t="s">
         <v>143</v>
       </c>
@@ -4160,7 +4172,7 @@
       <c r="E75" s="13"/>
       <c r="F75" s="13"/>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="19" t="s">
         <v>144</v>
       </c>
@@ -4172,7 +4184,7 @@
       <c r="E76" s="18"/>
       <c r="F76" s="18"/>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="19" t="s">
         <v>146</v>
       </c>
@@ -4184,7 +4196,7 @@
       <c r="E77" s="18"/>
       <c r="F77" s="18"/>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="19" t="s">
         <v>85</v>
       </c>
@@ -4196,7 +4208,7 @@
       <c r="E78" s="18"/>
       <c r="F78" s="18"/>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="19" t="s">
         <v>147</v>
       </c>
@@ -4208,7 +4220,7 @@
       <c r="E79" s="18"/>
       <c r="F79" s="18"/>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="19" t="s">
         <v>148</v>
       </c>
@@ -4220,7 +4232,7 @@
       <c r="E80" s="18"/>
       <c r="F80" s="18"/>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="19" t="s">
         <v>149</v>
       </c>
@@ -4232,7 +4244,7 @@
       <c r="E81" s="18"/>
       <c r="F81" s="18"/>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="19" t="s">
         <v>150</v>
       </c>
@@ -4244,7 +4256,7 @@
       <c r="E82" s="18"/>
       <c r="F82" s="18"/>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="19" t="s">
         <v>151</v>
       </c>
@@ -4256,7 +4268,7 @@
       <c r="E83" s="18"/>
       <c r="F83" s="18"/>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="19" t="s">
         <v>152</v>
       </c>
@@ -4268,7 +4280,7 @@
       <c r="E84" s="18"/>
       <c r="F84" s="18"/>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="19" t="s">
         <v>153</v>
       </c>
@@ -4280,7 +4292,7 @@
       <c r="E85" s="18"/>
       <c r="F85" s="18"/>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="18"/>
       <c r="B86" s="18"/>
       <c r="C86" s="18"/>
@@ -4302,25 +4314,25 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F88"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:F90"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.600000000000001" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>156</v>
       </c>
@@ -4340,7 +4352,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>158</v>
       </c>
@@ -4350,7 +4362,7 @@
       <c r="E5" s="23"/>
       <c r="F5" s="23"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>159</v>
       </c>
@@ -4371,7 +4383,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>161</v>
       </c>
@@ -4391,7 +4403,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>164</v>
       </c>
@@ -4400,18 +4412,18 @@
         <v>162</v>
       </c>
       <c r="D8" s="24">
-        <f>SUM(D69:D80)</f>
+        <f>SUM(D71:D82)</f>
         <v>230</v>
       </c>
       <c r="E8" s="24">
-        <f>SUM(E69:E80)</f>
+        <f>SUM(E71:E82)</f>
         <v>0</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>166</v>
       </c>
@@ -4431,7 +4443,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>168</v>
       </c>
@@ -4440,18 +4452,18 @@
         <v>162</v>
       </c>
       <c r="D10" s="27" t="str">
-        <f>IF(D8=0,"—",INDEX($A$69:$A$80,MATCH(MAX(D69:D80),D69:D80,0)))</f>
+        <f>IF(D8=0,"—",INDEX($A$71:$A$82,MATCH(MAX(D71:D82),D71:D82,0)))</f>
         <v>Cliente J</v>
       </c>
       <c r="E10" s="27" t="str">
-        <f>IF(E8=0,"—",INDEX($A$69:$A$80,MATCH(MAX(E69:E80),E69:E80,0)))</f>
+        <f>IF(E8=0,"—",INDEX($A$71:$A$82,MATCH(MAX(E71:E82),E71:E82,0)))</f>
         <v>—</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>170</v>
       </c>
@@ -4471,7 +4483,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>172</v>
       </c>
@@ -4492,7 +4504,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>174</v>
       </c>
@@ -4513,7 +4525,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>176</v>
       </c>
@@ -4534,7 +4546,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>178</v>
       </c>
@@ -4554,7 +4566,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
         <v>180</v>
       </c>
@@ -4564,7 +4576,7 @@
       <c r="E16" s="23"/>
       <c r="F16" s="23"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>181</v>
       </c>
@@ -4585,7 +4597,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>183</v>
       </c>
@@ -4605,7 +4617,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>185</v>
       </c>
@@ -4626,7 +4638,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>187</v>
       </c>
@@ -4647,7 +4659,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>189</v>
       </c>
@@ -4668,174 +4680,176 @@
         <v>190</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
+        <v>442</v>
+      </c>
+      <c r="B22" s="17"/>
+      <c r="C22" s="26">
+        <f>IF(C19&lt;=0,"n.d.",Input!C11/C19)</f>
+        <v>4.5592705167173252E-2</v>
+      </c>
+      <c r="D22" s="26">
+        <f>IF(D19&lt;=0,"n.d.",Input!D11/D19)</f>
+        <v>3.8194444444444448E-2</v>
+      </c>
+      <c r="E22" s="26">
+        <f>IF(E19&lt;=0,"n.d.",Input!E11/E19)</f>
+        <v>4.4858523119392688E-2</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
         <v>191</v>
       </c>
-      <c r="B22" s="17"/>
-      <c r="C22" s="25" t="s">
+      <c r="B23" s="17"/>
+      <c r="C23" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="D22" s="26">
+      <c r="D23" s="26">
         <f>IF(Input!C11=0,"n.d.",Input!D11/Input!C11-1)</f>
         <v>-8.333333333333337E-2</v>
       </c>
-      <c r="E22" s="26">
+      <c r="E23" s="26">
         <f>IF(Input!D11=0,"n.d.",Input!E11/Input!D11-1)</f>
         <v>0.18181818181818188</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A23" s="14" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="B23" s="17"/>
-      <c r="C23" s="24">
+      <c r="B24" s="17"/>
+      <c r="C24" s="24">
         <f>-Input!C44</f>
         <v>0</v>
       </c>
-      <c r="D23" s="24">
+      <c r="D24" s="24">
         <f>-Input!D44</f>
         <v>0</v>
       </c>
-      <c r="E23" s="24">
+      <c r="E24" s="24">
         <f>-Input!E44</f>
         <v>5</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A24" s="14" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="26">
-        <f>IF(C19&lt;=0,"n.d.",C23/C19)</f>
-        <v>0</v>
-      </c>
-      <c r="D24" s="26">
-        <f>IF(D19&lt;=0,"n.d.",D23/D19)</f>
-        <v>0</v>
-      </c>
-      <c r="E24" s="26">
-        <f>IF(E19&lt;=0,"n.d.",E23/E19)</f>
+      <c r="B25" s="17"/>
+      <c r="C25" s="26">
+        <f>IF(C19&lt;=0,"n.d.",C24/C19)</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="26">
+        <f>IF(D19&lt;=0,"n.d.",D24/D19)</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="26">
+        <f>IF(E19&lt;=0,"n.d.",E24/E19)</f>
         <v>3.450655624568668E-3</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F25" s="2" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A25" s="14" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="14" t="s">
         <v>197</v>
-      </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="24">
-        <f>C19-C23</f>
-        <v>1316</v>
-      </c>
-      <c r="D25" s="24">
-        <f>D19-D23</f>
-        <v>1440</v>
-      </c>
-      <c r="E25" s="24">
-        <f>E19-E23</f>
-        <v>1444</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A26" s="14" t="s">
-        <v>199</v>
       </c>
       <c r="B26" s="17"/>
       <c r="C26" s="24">
+        <f>C19-C24</f>
+        <v>1316</v>
+      </c>
+      <c r="D26" s="24">
+        <f>D19-D24</f>
+        <v>1440</v>
+      </c>
+      <c r="E26" s="24">
+        <f>E19-E24</f>
+        <v>1444</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="B27" s="17"/>
+      <c r="C27" s="24">
         <f>SUM(Input!C64:C68)</f>
         <v>25</v>
       </c>
-      <c r="D26" s="24">
+      <c r="D27" s="24">
         <f>SUM(Input!D64:D68)</f>
         <v>35</v>
       </c>
-      <c r="E26" s="24">
+      <c r="E27" s="24">
         <f>SUM(Input!E64:E68)</f>
         <v>40</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F27" s="2" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A27" s="14" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="14" t="s">
         <v>201</v>
       </c>
-      <c r="B27" s="17"/>
-      <c r="C27" s="24">
-        <f>C19+C26</f>
+      <c r="B28" s="17"/>
+      <c r="C28" s="24">
+        <f>C19+C27</f>
         <v>1341</v>
       </c>
-      <c r="D27" s="24">
-        <f>D19+D26</f>
+      <c r="D28" s="24">
+        <f>D19+D27</f>
         <v>1475</v>
       </c>
-      <c r="E27" s="24">
-        <f>E19+E26</f>
+      <c r="E28" s="24">
+        <f>E19+E27</f>
         <v>1489</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="F28" s="2" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A28" s="14" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="14" t="s">
         <v>203</v>
       </c>
-      <c r="B28" s="17"/>
-      <c r="C28" s="26">
-        <f>IF(C19&lt;=0,"n.d.",C26/C19)</f>
+      <c r="B29" s="17"/>
+      <c r="C29" s="26">
+        <f>IF(C19&lt;=0,"n.d.",C27/C19)</f>
         <v>1.8996960486322188E-2</v>
       </c>
-      <c r="D28" s="26">
-        <f>IF(D19&lt;=0,"n.d.",D26/D19)</f>
+      <c r="D29" s="26">
+        <f>IF(D19&lt;=0,"n.d.",D27/D19)</f>
         <v>2.4305555555555556E-2</v>
       </c>
-      <c r="E28" s="26">
-        <f>IF(E19&lt;=0,"n.d.",E26/E19)</f>
+      <c r="E29" s="26">
+        <f>IF(E19&lt;=0,"n.d.",E27/E19)</f>
         <v>2.7605244996549344E-2</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="F29" s="2" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A29" s="14" t="s">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="14" t="s">
         <v>205</v>
-      </c>
-      <c r="B29" s="17"/>
-      <c r="C29" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="D29" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="E29" s="29">
-        <f>SUM(E83:E87)</f>
-        <v>0</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A30" s="14" t="s">
-        <v>207</v>
       </c>
       <c r="B30" s="17"/>
       <c r="C30" s="25" t="s">
@@ -4844,509 +4858,511 @@
       <c r="D30" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="E30" s="27" t="str">
-        <f>IF(E29=0,"—",INDEX($A$83:$A$87,MATCH(1,E83:E87,0)))</f>
+      <c r="E30" s="29">
+        <f>SUM(E85:E89)</f>
+        <v>0</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="14" t="s">
+        <v>207</v>
+      </c>
+      <c r="B31" s="17"/>
+      <c r="C31" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="D31" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="E31" s="27" t="str">
+        <f>IF(E30=0,"—",INDEX($A$85:$A$89,MATCH(1,E85:E89,0)))</f>
         <v>—</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="F31" s="2" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A31" s="12" t="s">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
         <v>209</v>
       </c>
-      <c r="B31" s="23"/>
-      <c r="C31" s="23"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A32" s="14" t="s">
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="14" t="s">
         <v>210</v>
       </c>
-      <c r="B32" s="17"/>
-      <c r="C32" s="26">
+      <c r="B33" s="17"/>
+      <c r="C33" s="26">
         <f>Input!C22/Input!B22-1</f>
         <v>4.1129032258064413E-2</v>
       </c>
-      <c r="D32" s="26">
+      <c r="D33" s="26">
         <f>Input!D22/Input!C22-1</f>
         <v>4.5701006971339941E-2</v>
       </c>
-      <c r="E32" s="26">
+      <c r="E33" s="26">
         <f>Input!E22/Input!D22-1</f>
         <v>5.1851851851851816E-2</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="F33" s="2" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A33" s="14" t="s">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="14" t="s">
         <v>212</v>
       </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="25" t="s">
+      <c r="B34" s="17"/>
+      <c r="C34" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="D33" s="28">
-        <f>(D32-D7)*100</f>
+      <c r="D34" s="28">
+        <f>(D33-D7)*100</f>
         <v>-3.5162460760740366E-2</v>
       </c>
-      <c r="E33" s="28">
-        <f>(E32-E7)*100</f>
+      <c r="E34" s="28">
+        <f>(E33-E7)*100</f>
         <v>0.15373864430467954</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="F34" s="2" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A34" s="14" t="s">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="14" t="s">
         <v>214</v>
       </c>
-      <c r="B34" s="17"/>
-      <c r="C34" s="30">
+      <c r="B35" s="17"/>
+      <c r="C35" s="30">
         <f>Input!C22/C6*365</f>
         <v>62.001973684210526</v>
       </c>
-      <c r="D34" s="30">
+      <c r="D35" s="30">
         <f>Input!D22/D6*365</f>
         <v>61.981132075471692</v>
       </c>
-      <c r="E34" s="30">
+      <c r="E35" s="30">
         <f>Input!E22/E6*365</f>
         <v>62.071856287425149</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="F35" s="2" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A35" s="14" t="s">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="14" t="s">
         <v>216</v>
       </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="25" t="s">
+      <c r="B36" s="17"/>
+      <c r="C36" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="D35" s="30">
-        <f>D34-C34</f>
+      <c r="D36" s="30">
+        <f>D35-C35</f>
         <v>-2.0841608738834339E-2</v>
       </c>
-      <c r="E35" s="30">
-        <f>E34-D34</f>
+      <c r="E36" s="30">
+        <f>E35-D35</f>
         <v>9.0724211953457257E-2</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="F36" s="2" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A36" s="14" t="s">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="14" t="s">
         <v>218</v>
       </c>
-      <c r="B36" s="17"/>
-      <c r="C36" s="26">
+      <c r="B37" s="17"/>
+      <c r="C37" s="26">
         <f>Input!C21/Input!B21-1</f>
         <v>3.6866359447004671E-2</v>
       </c>
-      <c r="D36" s="26">
+      <c r="D37" s="26">
         <f>Input!D21/Input!C21-1</f>
         <v>4.0000000000000036E-2</v>
       </c>
-      <c r="E36" s="26">
+      <c r="E37" s="26">
         <f>Input!E21/Input!D21-1</f>
         <v>5.555555555555558E-2</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="F37" s="2" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A37" s="14" t="s">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="14" t="s">
         <v>220</v>
-      </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="D37" s="26">
-        <f>Input!D7/Input!C7-1</f>
-        <v>4.0296052631578982E-2</v>
-      </c>
-      <c r="E37" s="26">
-        <f>Input!E7/Input!D7-1</f>
-        <v>5.7619675010979421E-2</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A38" s="14" t="s">
-        <v>222</v>
       </c>
       <c r="B38" s="17"/>
       <c r="C38" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="D38" s="28">
-        <f>(D36-D37)*100</f>
+      <c r="D38" s="26">
+        <f>Input!D7/Input!C7-1</f>
+        <v>4.0296052631578982E-2</v>
+      </c>
+      <c r="E38" s="26">
+        <f>Input!E7/Input!D7-1</f>
+        <v>5.7619675010979421E-2</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="B39" s="17"/>
+      <c r="C39" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="D39" s="28">
+        <f>(D37-D38)*100</f>
         <v>-2.960526315789469E-2</v>
       </c>
-      <c r="E38" s="28">
-        <f>(E36-E37)*100</f>
+      <c r="E39" s="28">
+        <f>(E37-E38)*100</f>
         <v>-0.20641194554238407</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="F39" s="2" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A39" s="14" t="s">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="B39" s="17"/>
-      <c r="C39" s="30">
+      <c r="B40" s="17"/>
+      <c r="C40" s="30">
         <f>Input!C21/-Input!C7*365</f>
         <v>75.04111842105263</v>
       </c>
-      <c r="D39" s="30">
+      <c r="D40" s="30">
         <f>Input!D21/-Input!D7*365</f>
         <v>75.019762845849812</v>
       </c>
-      <c r="E39" s="30">
+      <c r="E40" s="30">
         <f>Input!E21/-Input!E7*365</f>
         <v>74.873349389585584</v>
       </c>
-      <c r="F39" s="2" t="s">
+      <c r="F40" s="2" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A40" s="14" t="s">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="14" t="s">
         <v>226</v>
       </c>
-      <c r="B40" s="17"/>
-      <c r="C40" s="30">
+      <c r="B41" s="17"/>
+      <c r="C41" s="30">
         <f>Input!C29/-Input!C7*365</f>
         <v>60.03289473684211</v>
       </c>
-      <c r="D40" s="30">
+      <c r="D41" s="30">
         <f>Input!D29/-Input!D7*365</f>
         <v>59.951690821256044</v>
       </c>
-      <c r="E40" s="30">
+      <c r="E41" s="30">
         <f>Input!E29/-Input!E7*365</f>
         <v>60.019931899343909</v>
       </c>
-      <c r="F40" s="2" t="s">
+      <c r="F41" s="2" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A41" s="14" t="s">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="14" t="s">
         <v>228</v>
       </c>
-      <c r="B41" s="17"/>
-      <c r="C41" s="25" t="s">
+      <c r="B42" s="17"/>
+      <c r="C42" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="D41" s="30">
-        <f>D40-C40</f>
+      <c r="D42" s="30">
+        <f>D41-C41</f>
         <v>-8.1203915586065989E-2</v>
       </c>
-      <c r="E41" s="30">
-        <f>E40-D40</f>
+      <c r="E42" s="30">
+        <f>E41-D41</f>
         <v>6.8241078087865503E-2</v>
       </c>
-      <c r="F41" s="2" t="s">
+      <c r="F42" s="2" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A42" s="12" t="s">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="12" t="s">
         <v>230</v>
       </c>
-      <c r="B42" s="23"/>
-      <c r="C42" s="23"/>
-      <c r="D42" s="23"/>
-      <c r="E42" s="23"/>
-      <c r="F42" s="23"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A43" s="14" t="s">
+      <c r="B43" s="23"/>
+      <c r="C43" s="23"/>
+      <c r="D43" s="23"/>
+      <c r="E43" s="23"/>
+      <c r="F43" s="23"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="14" t="s">
         <v>231</v>
       </c>
-      <c r="B43" s="17"/>
-      <c r="C43" s="24">
+      <c r="B44" s="17"/>
+      <c r="C44" s="24">
         <f>Input!C40</f>
         <v>1194</v>
       </c>
-      <c r="D43" s="24">
+      <c r="D44" s="24">
         <f>Input!D40</f>
         <v>1312</v>
       </c>
-      <c r="E43" s="24">
+      <c r="E44" s="24">
         <f>Input!E40</f>
         <v>1294</v>
       </c>
-      <c r="F43" s="2" t="s">
+      <c r="F44" s="2" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A44" s="14" t="s">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="B44" s="17"/>
-      <c r="C44" s="26">
-        <f>IF(C19&lt;=0,"n.d.",C43/C19)</f>
+      <c r="B45" s="17"/>
+      <c r="C45" s="26">
+        <f>IF(C19&lt;=0,"n.d.",C44/C19)</f>
         <v>0.90729483282674772</v>
       </c>
-      <c r="D44" s="26">
-        <f>IF(D19&lt;=0,"n.d.",D43/D19)</f>
+      <c r="D45" s="26">
+        <f>IF(D19&lt;=0,"n.d.",D44/D19)</f>
         <v>0.91111111111111109</v>
       </c>
-      <c r="E44" s="26">
-        <f>IF(E19&lt;=0,"n.d.",E43/E19)</f>
+      <c r="E45" s="26">
+        <f>IF(E19&lt;=0,"n.d.",E44/E19)</f>
         <v>0.89302967563837132</v>
       </c>
-      <c r="F44" s="2" t="s">
+      <c r="F45" s="2" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A45" s="14" t="s">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="14" t="s">
+        <v>444</v>
+      </c>
+      <c r="B46" s="17"/>
+      <c r="C46" s="26">
+        <f>IF(SUM($C$19:C19)&lt;=0,"n.d.",SUM($C$44:C44)/SUM($C$19:C19))</f>
+        <v>0.90729483282674772</v>
+      </c>
+      <c r="D46" s="26">
+        <f>IF(SUM($C$19:D19)&lt;=0,"n.d.",SUM($C$44:D44)/SUM($C$19:D19))</f>
+        <v>0.90928882438316405</v>
+      </c>
+      <c r="E46" s="26">
+        <f>IF(SUM($C$19:E19)&lt;=0,"n.d.",SUM($C$44:E44)/SUM($C$19:E19))</f>
+        <v>0.90368608799048755</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="14" t="s">
         <v>235</v>
       </c>
-      <c r="B45" s="17"/>
-      <c r="C45" s="24">
+      <c r="B47" s="17"/>
+      <c r="C47" s="24">
         <f>Input!C41</f>
         <v>882</v>
       </c>
-      <c r="D45" s="24">
+      <c r="D47" s="24">
         <f>Input!D41</f>
         <v>986</v>
       </c>
-      <c r="E45" s="24">
+      <c r="E47" s="24">
         <f>Input!E41</f>
         <v>985</v>
       </c>
-      <c r="F45" s="2" t="s">
+      <c r="F47" s="2" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A46" s="14" t="s">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="14" t="s">
         <v>237</v>
       </c>
-      <c r="B46" s="17"/>
-      <c r="C46" s="24">
+      <c r="B48" s="17"/>
+      <c r="C48" s="24">
         <f>Input!C41+Input!C42+Input!C43</f>
         <v>552</v>
       </c>
-      <c r="D46" s="24">
+      <c r="D48" s="24">
         <f>Input!D41+Input!D42+Input!D43</f>
         <v>636</v>
       </c>
-      <c r="E46" s="24">
+      <c r="E48" s="24">
         <f>Input!E41+Input!E42+Input!E43</f>
         <v>625</v>
       </c>
-      <c r="F46" s="2" t="s">
+      <c r="F48" s="2" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A47" s="14" t="s">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="14" t="s">
         <v>239</v>
       </c>
-      <c r="B47" s="17"/>
-      <c r="C47" s="26">
+      <c r="B49" s="17"/>
+      <c r="C49" s="26">
         <f>-Input!C42/C6</f>
         <v>2.1710526315789475E-2</v>
       </c>
-      <c r="D47" s="26">
+      <c r="D49" s="26">
         <f>-Input!D42/D6</f>
         <v>2.20125786163522E-2</v>
       </c>
-      <c r="E47" s="26">
+      <c r="E49" s="26">
         <f>-Input!E42/E6</f>
         <v>2.2754491017964073E-2</v>
       </c>
-      <c r="F47" s="2" t="s">
+      <c r="F49" s="2" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A48" s="12" t="s">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="B48" s="23"/>
-      <c r="C48" s="23"/>
-      <c r="D48" s="23"/>
-      <c r="E48" s="23"/>
-      <c r="F48" s="23"/>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A49" s="14" t="s">
+      <c r="B50" s="23"/>
+      <c r="C50" s="23"/>
+      <c r="D50" s="23"/>
+      <c r="E50" s="23"/>
+      <c r="F50" s="23"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="14" t="s">
         <v>242</v>
       </c>
-      <c r="B49" s="24">
+      <c r="B51" s="24">
         <f>Input!B27+Input!B30</f>
         <v>2400</v>
       </c>
-      <c r="C49" s="24">
+      <c r="C51" s="24">
         <f>Input!C27+Input!C30</f>
         <v>2040</v>
       </c>
-      <c r="D49" s="24">
+      <c r="D51" s="24">
         <f>Input!D27+Input!D30</f>
         <v>1680</v>
       </c>
-      <c r="E49" s="24">
+      <c r="E51" s="24">
         <f>Input!E27+Input!E30</f>
         <v>1320</v>
       </c>
-      <c r="F49" s="2" t="s">
+      <c r="F51" s="2" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A50" s="14" t="s">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="14" t="s">
         <v>244</v>
       </c>
-      <c r="B50" s="26">
-        <f>IF(B49=0,"n.d.",Input!B30/B49)</f>
+      <c r="B52" s="26">
+        <f>IF(B51=0,"n.d.",Input!B30/B51)</f>
         <v>0.15</v>
       </c>
-      <c r="C50" s="26">
-        <f>IF(C49=0,"n.d.",Input!C30/C49)</f>
+      <c r="C52" s="26">
+        <f>IF(C51=0,"n.d.",Input!C30/C51)</f>
         <v>0.17647058823529413</v>
       </c>
-      <c r="D50" s="26">
-        <f>IF(D49=0,"n.d.",Input!D30/D49)</f>
+      <c r="D52" s="26">
+        <f>IF(D51=0,"n.d.",Input!D30/D51)</f>
         <v>0.21428571428571427</v>
       </c>
-      <c r="E50" s="26">
-        <f>IF(E49=0,"n.d.",Input!E30/E49)</f>
+      <c r="E52" s="26">
+        <f>IF(E51=0,"n.d.",Input!E30/E51)</f>
         <v>0.27272727272727271</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="F52" s="2" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A51" s="14" t="s">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="14" t="s">
         <v>246</v>
       </c>
-      <c r="B51" s="24">
-        <f>B49-Input!B24</f>
+      <c r="B53" s="24">
+        <f>B51-Input!B24</f>
         <v>1700</v>
       </c>
-      <c r="C51" s="24">
-        <f>C49-Input!C24</f>
+      <c r="C53" s="24">
+        <f>C51-Input!C24</f>
         <v>1398</v>
       </c>
-      <c r="D51" s="24">
-        <f>D49-Input!D24</f>
+      <c r="D53" s="24">
+        <f>D51-Input!D24</f>
         <v>1062</v>
       </c>
-      <c r="E51" s="24">
-        <f>E49-Input!E24</f>
+      <c r="E53" s="24">
+        <f>E51-Input!E24</f>
         <v>767</v>
       </c>
-      <c r="F51" s="2" t="s">
+      <c r="F53" s="2" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A52" s="14" t="s">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="14" t="s">
         <v>248</v>
       </c>
-      <c r="B52" s="17"/>
-      <c r="C52" s="31">
-        <f>IF(C19&lt;=0,"n.d.",C51/C19)</f>
+      <c r="B54" s="17"/>
+      <c r="C54" s="31">
+        <f>IF(C19&lt;=0,"n.d.",C53/C19)</f>
         <v>1.0623100303951367</v>
       </c>
-      <c r="D52" s="31">
-        <f>IF(D19&lt;=0,"n.d.",D51/D19)</f>
+      <c r="D54" s="31">
+        <f>IF(D19&lt;=0,"n.d.",D53/D19)</f>
         <v>0.73750000000000004</v>
       </c>
-      <c r="E52" s="31">
-        <f>IF(E19&lt;=0,"n.d.",E51/E19)</f>
+      <c r="E54" s="31">
+        <f>IF(E19&lt;=0,"n.d.",E53/E19)</f>
         <v>0.52933057280883367</v>
       </c>
-      <c r="F52" s="2" t="s">
+      <c r="F54" s="2" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A53" s="14" t="s">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="14" t="s">
         <v>250</v>
       </c>
-      <c r="B53" s="17"/>
-      <c r="C53" s="31">
-        <f>IF(C25&lt;=0,"n.d.",C51/C25)</f>
+      <c r="B55" s="17"/>
+      <c r="C55" s="31">
+        <f>IF(C26&lt;=0,"n.d.",C53/C26)</f>
         <v>1.0623100303951367</v>
       </c>
-      <c r="D53" s="31">
-        <f>IF(D25&lt;=0,"n.d.",D51/D25)</f>
+      <c r="D55" s="31">
+        <f>IF(D26&lt;=0,"n.d.",D53/D26)</f>
         <v>0.73750000000000004</v>
       </c>
-      <c r="E53" s="31">
-        <f>IF(E25&lt;=0,"n.d.",E51/E25)</f>
+      <c r="E55" s="31">
+        <f>IF(E26&lt;=0,"n.d.",E53/E26)</f>
         <v>0.53116343490304707</v>
       </c>
-      <c r="F53" s="2" t="s">
+      <c r="F55" s="2" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A54" s="14" t="s">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="14" t="s">
         <v>252</v>
-      </c>
-      <c r="B54" s="17"/>
-      <c r="C54" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="D54" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="E54" s="31">
-        <f>Input!E73</f>
-        <v>3</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A55" s="14" t="s">
-        <v>254</v>
-      </c>
-      <c r="B55" s="17"/>
-      <c r="C55" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="D55" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="E55" s="26">
-        <f>IF(ISNUMBER(E52),1-E52/E54,"n.d.")</f>
-        <v>0.82355647573038882</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A56" s="14" t="s">
-        <v>256</v>
       </c>
       <c r="B56" s="17"/>
       <c r="C56" s="25" t="s">
@@ -5355,164 +5371,173 @@
       <c r="D56" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="E56" s="24">
-        <f>E51/E54</f>
+      <c r="E56" s="31">
+        <f>Input!E73</f>
+        <v>3</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="B57" s="17"/>
+      <c r="C57" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="D57" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="E57" s="26">
+        <f>IF(ISNUMBER(E54),1-E54/E56,"n.d.")</f>
+        <v>0.82355647573038882</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="B58" s="17"/>
+      <c r="C58" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="D58" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="E58" s="24">
+        <f>E53/E56</f>
         <v>255.66666666666666</v>
       </c>
-      <c r="F56" s="2" t="s">
+      <c r="F58" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A57" s="12" t="s">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="12" t="s">
         <v>258</v>
       </c>
-      <c r="B57" s="23"/>
-      <c r="C57" s="23"/>
-      <c r="D57" s="23"/>
-      <c r="E57" s="23"/>
-      <c r="F57" s="23"/>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A58" s="14" t="s">
+      <c r="B59" s="23"/>
+      <c r="C59" s="23"/>
+      <c r="D59" s="23"/>
+      <c r="E59" s="23"/>
+      <c r="F59" s="23"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="14" t="s">
         <v>259</v>
       </c>
-      <c r="B58" s="24">
+      <c r="B60" s="24">
         <f>(Input!B19+Input!B20+Input!B21+Input!B22+Input!B23+Input!B24)-(Input!B25+Input!B27+Input!B28+Input!B29+Input!B30+Input!B31)</f>
         <v>0</v>
       </c>
-      <c r="C58" s="24">
+      <c r="C60" s="24">
         <f>(Input!C19+Input!C20+Input!C21+Input!C22+Input!C23+Input!C24)-(Input!C25+Input!C27+Input!C28+Input!C29+Input!C30+Input!C31)</f>
         <v>0</v>
       </c>
-      <c r="D58" s="24">
+      <c r="D60" s="24">
         <f>(Input!D19+Input!D20+Input!D21+Input!D22+Input!D23+Input!D24)-(Input!D25+Input!D27+Input!D28+Input!D29+Input!D30+Input!D31)</f>
         <v>0</v>
       </c>
-      <c r="E58" s="24">
+      <c r="E60" s="24">
         <f>(Input!E19+Input!E20+Input!E21+Input!E22+Input!E23+Input!E24)-(Input!E25+Input!E27+Input!E28+Input!E29+Input!E30+Input!E31)</f>
         <v>0</v>
       </c>
-      <c r="F58" s="2" t="s">
+      <c r="F60" s="2" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A59" s="14" t="s">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="14" t="s">
         <v>261</v>
-      </c>
-      <c r="B59" s="17"/>
-      <c r="C59" s="24">
-        <f>Input!C46-Input!C24</f>
-        <v>0</v>
-      </c>
-      <c r="D59" s="24">
-        <f>Input!D46-Input!D24</f>
-        <v>0</v>
-      </c>
-      <c r="E59" s="24">
-        <f>Input!E46-Input!E24</f>
-        <v>0</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A60" s="14" t="s">
-        <v>262</v>
-      </c>
-      <c r="B60" s="17"/>
-      <c r="C60" s="24">
-        <f>ABS(Input!C35+(Input!C22-Input!B22))+ABS(Input!C36+(Input!C21-Input!B21))+ABS(Input!C37-(Input!C29-Input!B29))+ABS(Input!C38+(Input!C23-Input!B23))+ABS(Input!C39-(Input!C31-Input!B31))</f>
-        <v>0</v>
-      </c>
-      <c r="D60" s="24">
-        <f>ABS(Input!D35+(Input!D22-Input!C22))+ABS(Input!D36+(Input!D21-Input!C21))+ABS(Input!D37-(Input!D29-Input!C29))+ABS(Input!D38+(Input!D23-Input!C23))+ABS(Input!D39-(Input!D31-Input!C31))</f>
-        <v>0</v>
-      </c>
-      <c r="E60" s="24">
-        <f>ABS(Input!E35+(Input!E22-Input!D22))+ABS(Input!E36+(Input!E21-Input!D21))+ABS(Input!E37-(Input!E29-Input!D29))+ABS(Input!E38+(Input!E23-Input!D23))+ABS(Input!E39-(Input!E31-Input!D31))</f>
-        <v>0</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A61" s="14" t="s">
-        <v>264</v>
       </c>
       <c r="B61" s="17"/>
       <c r="C61" s="24">
-        <f>MAX(ABS(Input!C16-Input!C26),ABS(Input!C16-Input!C34))</f>
+        <f>Input!C46-Input!C24</f>
         <v>0</v>
       </c>
       <c r="D61" s="24">
-        <f>MAX(ABS(Input!D16-Input!D26),ABS(Input!D16-Input!D34))</f>
+        <f>Input!D46-Input!D24</f>
         <v>0</v>
       </c>
       <c r="E61" s="24">
-        <f>MAX(ABS(Input!E16-Input!E26),ABS(Input!E16-Input!E34))</f>
+        <f>Input!E46-Input!E24</f>
         <v>0</v>
       </c>
       <c r="F61" s="2" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="14" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B62" s="17"/>
       <c r="C62" s="24">
+        <f>ABS(Input!C35+(Input!C22-Input!B22))+ABS(Input!C36+(Input!C21-Input!B21))+ABS(Input!C37-(Input!C29-Input!B29))+ABS(Input!C38+(Input!C23-Input!B23))+ABS(Input!C39-(Input!C31-Input!B31))</f>
+        <v>0</v>
+      </c>
+      <c r="D62" s="24">
+        <f>ABS(Input!D35+(Input!D22-Input!C22))+ABS(Input!D36+(Input!D21-Input!C21))+ABS(Input!D37-(Input!D29-Input!C29))+ABS(Input!D38+(Input!D23-Input!C23))+ABS(Input!D39-(Input!D31-Input!C31))</f>
+        <v>0</v>
+      </c>
+      <c r="E62" s="24">
+        <f>ABS(Input!E35+(Input!E22-Input!D22))+ABS(Input!E36+(Input!E21-Input!D21))+ABS(Input!E37-(Input!E29-Input!D29))+ABS(Input!E38+(Input!E23-Input!D23))+ABS(Input!E39-(Input!E31-Input!D31))</f>
+        <v>0</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="14" t="s">
+        <v>264</v>
+      </c>
+      <c r="B63" s="17"/>
+      <c r="C63" s="24">
+        <f>MAX(ABS(Input!C16-Input!C26),ABS(Input!C16-Input!C34))</f>
+        <v>0</v>
+      </c>
+      <c r="D63" s="24">
+        <f>MAX(ABS(Input!D16-Input!D26),ABS(Input!D16-Input!D34))</f>
+        <v>0</v>
+      </c>
+      <c r="E63" s="24">
+        <f>MAX(ABS(Input!E16-Input!E26),ABS(Input!E16-Input!E34))</f>
+        <v>0</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="B64" s="17"/>
+      <c r="C64" s="24">
         <f>SUM(Input!C49:C61)-C6</f>
         <v>0</v>
       </c>
-      <c r="D62" s="24">
+      <c r="D64" s="24">
         <f>SUM(Input!D49:D61)-D6</f>
         <v>0</v>
       </c>
-      <c r="E62" s="24">
+      <c r="E64" s="24">
         <f>SUM(Input!E49:E61)-E6</f>
         <v>0</v>
       </c>
-      <c r="F62" s="2" t="s">
+      <c r="F64" s="2" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A63" s="14" t="s">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="14" t="s">
         <v>266</v>
-      </c>
-      <c r="B63" s="17"/>
-      <c r="C63" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="D63" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="E63" s="24">
-        <f>ABS(Input!E71-E49)+ABS(Input!E72-Input!E30)</f>
-        <v>0</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A64" s="12" t="s">
-        <v>268</v>
-      </c>
-      <c r="B64" s="23"/>
-      <c r="C64" s="23"/>
-      <c r="D64" s="23"/>
-      <c r="E64" s="23"/>
-      <c r="F64" s="23"/>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A65" s="14" t="s">
-        <v>269</v>
       </c>
       <c r="B65" s="17"/>
       <c r="C65" s="25" t="s">
@@ -5521,374 +5546,403 @@
       <c r="D65" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="E65" s="29">
+      <c r="E65" s="24">
+        <f>ABS(Input!E71-E51)+ABS(Input!E72-Input!E30)</f>
+        <v>0</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="B66" s="23"/>
+      <c r="C66" s="23"/>
+      <c r="D66" s="23"/>
+      <c r="E66" s="23"/>
+      <c r="F66" s="23"/>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="B67" s="17"/>
+      <c r="C67" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="D67" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="E67" s="29">
         <f>COUNTIF(Input!B76:B85,"Não")</f>
         <v>0</v>
       </c>
-      <c r="F65" s="2" t="s">
+      <c r="F67" s="2" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A66" s="14" t="s">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="14" t="s">
         <v>271</v>
       </c>
-      <c r="B66" s="17"/>
-      <c r="C66" s="25" t="s">
+      <c r="B68" s="17"/>
+      <c r="C68" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="D66" s="25" t="s">
+      <c r="D68" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="E66" s="27" t="str">
+      <c r="E68" s="27" t="str">
         <f>IF(LEN(IF(Input!B76="Não",Input!A76&amp;"; ","")&amp;IF(Input!B77="Não",Input!A77&amp;"; ","")&amp;IF(Input!B78="Não",Input!A78&amp;"; ","")&amp;IF(Input!B79="Não",Input!A79&amp;"; ","")&amp;IF(Input!B80="Não",Input!A80&amp;"; ","")&amp;IF(Input!B81="Não",Input!A81&amp;"; ","")&amp;IF(Input!B82="Não",Input!A82&amp;"; ","")&amp;IF(Input!B83="Não",Input!A83&amp;"; ","")&amp;IF(Input!B84="Não",Input!A84&amp;"; ","")&amp;IF(Input!B85="Não",Input!A85&amp;"; ",""))=0,"—",LEFT(IF(Input!B76="Não",Input!A76&amp;"; ","")&amp;IF(Input!B77="Não",Input!A77&amp;"; ","")&amp;IF(Input!B78="Não",Input!A78&amp;"; ","")&amp;IF(Input!B79="Não",Input!A79&amp;"; ","")&amp;IF(Input!B80="Não",Input!A80&amp;"; ","")&amp;IF(Input!B81="Não",Input!A81&amp;"; ","")&amp;IF(Input!B82="Não",Input!A82&amp;"; ","")&amp;IF(Input!B83="Não",Input!A83&amp;"; ","")&amp;IF(Input!B84="Não",Input!A84&amp;"; ","")&amp;IF(Input!B85="Não",Input!A85&amp;"; ",""),LEN(IF(Input!B76="Não",Input!A76&amp;"; ","")&amp;IF(Input!B77="Não",Input!A77&amp;"; ","")&amp;IF(Input!B78="Não",Input!A78&amp;"; ","")&amp;IF(Input!B79="Não",Input!A79&amp;"; ","")&amp;IF(Input!B80="Não",Input!A80&amp;"; ","")&amp;IF(Input!B81="Não",Input!A81&amp;"; ","")&amp;IF(Input!B82="Não",Input!A82&amp;"; ","")&amp;IF(Input!B83="Não",Input!A83&amp;"; ","")&amp;IF(Input!B84="Não",Input!A84&amp;"; ","")&amp;IF(Input!B85="Não",Input!A85&amp;"; ",""))-2))</f>
         <v>—</v>
       </c>
-      <c r="F66" s="2" t="s">
+      <c r="F68" s="2" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A67" s="32"/>
-      <c r="B67" s="32"/>
-      <c r="C67" s="32"/>
-      <c r="D67" s="32"/>
-      <c r="E67" s="32"/>
-      <c r="F67" s="32"/>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A68" s="12" t="s">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="32"/>
+      <c r="B69" s="32"/>
+      <c r="C69" s="32"/>
+      <c r="D69" s="32"/>
+      <c r="E69" s="32"/>
+      <c r="F69" s="32"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="12" t="s">
         <v>273</v>
       </c>
-      <c r="B68" s="23"/>
-      <c r="C68" s="23"/>
-      <c r="D68" s="23"/>
-      <c r="E68" s="23"/>
-      <c r="F68" s="23"/>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A69" s="33" t="str">
+      <c r="B70" s="23"/>
+      <c r="C70" s="23"/>
+      <c r="D70" s="23"/>
+      <c r="E70" s="23"/>
+      <c r="F70" s="23"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="33" t="str">
         <f>IF(Input!A49="","",Input!A49)</f>
         <v>Cliente A</v>
-      </c>
-      <c r="B69" s="32"/>
-      <c r="C69" s="34" t="s">
-        <v>162</v>
-      </c>
-      <c r="D69" s="35">
-        <f>IF(AND(N(Input!C49)=0,N(Input!D49)&gt;0),Input!D49,0)</f>
-        <v>0</v>
-      </c>
-      <c r="E69" s="35">
-        <f>IF(AND(N(Input!D49)=0,N(Input!E49)&gt;0),Input!E49,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F69" s="32"/>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A70" s="33" t="str">
-        <f>IF(Input!A50="","",Input!A50)</f>
-        <v>Cliente B</v>
-      </c>
-      <c r="B70" s="32"/>
-      <c r="C70" s="34" t="s">
-        <v>162</v>
-      </c>
-      <c r="D70" s="35">
-        <f>IF(AND(N(Input!C50)=0,N(Input!D50)&gt;0),Input!D50,0)</f>
-        <v>0</v>
-      </c>
-      <c r="E70" s="35">
-        <f>IF(AND(N(Input!D50)=0,N(Input!E50)&gt;0),Input!E50,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F70" s="32"/>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A71" s="33" t="str">
-        <f>IF(Input!A51="","",Input!A51)</f>
-        <v>Cliente C</v>
       </c>
       <c r="B71" s="32"/>
       <c r="C71" s="34" t="s">
         <v>162</v>
       </c>
       <c r="D71" s="35">
-        <f>IF(AND(N(Input!C51)=0,N(Input!D51)&gt;0),Input!D51,0)</f>
+        <f>IF(AND(N(Input!C49)=0,N(Input!D49)&gt;0),Input!D49,0)</f>
         <v>0</v>
       </c>
       <c r="E71" s="35">
-        <f>IF(AND(N(Input!D51)=0,N(Input!E51)&gt;0),Input!E51,0)</f>
+        <f>IF(AND(N(Input!D49)=0,N(Input!E49)&gt;0),Input!E49,0)</f>
         <v>0</v>
       </c>
       <c r="F71" s="32"/>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="33" t="str">
-        <f>IF(Input!A52="","",Input!A52)</f>
-        <v>Cliente D</v>
+        <f>IF(Input!A50="","",Input!A50)</f>
+        <v>Cliente B</v>
       </c>
       <c r="B72" s="32"/>
       <c r="C72" s="34" t="s">
         <v>162</v>
       </c>
       <c r="D72" s="35">
-        <f>IF(AND(N(Input!C52)=0,N(Input!D52)&gt;0),Input!D52,0)</f>
+        <f>IF(AND(N(Input!C50)=0,N(Input!D50)&gt;0),Input!D50,0)</f>
         <v>0</v>
       </c>
       <c r="E72" s="35">
-        <f>IF(AND(N(Input!D52)=0,N(Input!E52)&gt;0),Input!E52,0)</f>
+        <f>IF(AND(N(Input!D50)=0,N(Input!E50)&gt;0),Input!E50,0)</f>
         <v>0</v>
       </c>
       <c r="F72" s="32"/>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="33" t="str">
-        <f>IF(Input!A53="","",Input!A53)</f>
-        <v>Cliente E</v>
+        <f>IF(Input!A51="","",Input!A51)</f>
+        <v>Cliente C</v>
       </c>
       <c r="B73" s="32"/>
       <c r="C73" s="34" t="s">
         <v>162</v>
       </c>
       <c r="D73" s="35">
-        <f>IF(AND(N(Input!C53)=0,N(Input!D53)&gt;0),Input!D53,0)</f>
+        <f>IF(AND(N(Input!C51)=0,N(Input!D51)&gt;0),Input!D51,0)</f>
         <v>0</v>
       </c>
       <c r="E73" s="35">
-        <f>IF(AND(N(Input!D53)=0,N(Input!E53)&gt;0),Input!E53,0)</f>
+        <f>IF(AND(N(Input!D51)=0,N(Input!E51)&gt;0),Input!E51,0)</f>
         <v>0</v>
       </c>
       <c r="F73" s="32"/>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="33" t="str">
-        <f>IF(Input!A54="","",Input!A54)</f>
-        <v>Cliente F</v>
+        <f>IF(Input!A52="","",Input!A52)</f>
+        <v>Cliente D</v>
       </c>
       <c r="B74" s="32"/>
       <c r="C74" s="34" t="s">
         <v>162</v>
       </c>
       <c r="D74" s="35">
-        <f>IF(AND(N(Input!C54)=0,N(Input!D54)&gt;0),Input!D54,0)</f>
+        <f>IF(AND(N(Input!C52)=0,N(Input!D52)&gt;0),Input!D52,0)</f>
         <v>0</v>
       </c>
       <c r="E74" s="35">
-        <f>IF(AND(N(Input!D54)=0,N(Input!E54)&gt;0),Input!E54,0)</f>
+        <f>IF(AND(N(Input!D52)=0,N(Input!E52)&gt;0),Input!E52,0)</f>
         <v>0</v>
       </c>
       <c r="F74" s="32"/>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="33" t="str">
-        <f>IF(Input!A55="","",Input!A55)</f>
-        <v>Cliente G</v>
+        <f>IF(Input!A53="","",Input!A53)</f>
+        <v>Cliente E</v>
       </c>
       <c r="B75" s="32"/>
       <c r="C75" s="34" t="s">
         <v>162</v>
       </c>
       <c r="D75" s="35">
-        <f>IF(AND(N(Input!C55)=0,N(Input!D55)&gt;0),Input!D55,0)</f>
+        <f>IF(AND(N(Input!C53)=0,N(Input!D53)&gt;0),Input!D53,0)</f>
         <v>0</v>
       </c>
       <c r="E75" s="35">
-        <f>IF(AND(N(Input!D55)=0,N(Input!E55)&gt;0),Input!E55,0)</f>
+        <f>IF(AND(N(Input!D53)=0,N(Input!E53)&gt;0),Input!E53,0)</f>
         <v>0</v>
       </c>
       <c r="F75" s="32"/>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="33" t="str">
-        <f>IF(Input!A56="","",Input!A56)</f>
-        <v>Cliente H</v>
+        <f>IF(Input!A54="","",Input!A54)</f>
+        <v>Cliente F</v>
       </c>
       <c r="B76" s="32"/>
       <c r="C76" s="34" t="s">
         <v>162</v>
       </c>
       <c r="D76" s="35">
-        <f>IF(AND(N(Input!C56)=0,N(Input!D56)&gt;0),Input!D56,0)</f>
+        <f>IF(AND(N(Input!C54)=0,N(Input!D54)&gt;0),Input!D54,0)</f>
         <v>0</v>
       </c>
       <c r="E76" s="35">
-        <f>IF(AND(N(Input!D56)=0,N(Input!E56)&gt;0),Input!E56,0)</f>
+        <f>IF(AND(N(Input!D54)=0,N(Input!E54)&gt;0),Input!E54,0)</f>
         <v>0</v>
       </c>
       <c r="F76" s="32"/>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="33" t="str">
-        <f>IF(Input!A57="","",Input!A57)</f>
-        <v>Cliente I</v>
+        <f>IF(Input!A55="","",Input!A55)</f>
+        <v>Cliente G</v>
       </c>
       <c r="B77" s="32"/>
       <c r="C77" s="34" t="s">
         <v>162</v>
       </c>
       <c r="D77" s="35">
-        <f>IF(AND(N(Input!C57)=0,N(Input!D57)&gt;0),Input!D57,0)</f>
+        <f>IF(AND(N(Input!C55)=0,N(Input!D55)&gt;0),Input!D55,0)</f>
         <v>0</v>
       </c>
       <c r="E77" s="35">
-        <f>IF(AND(N(Input!D57)=0,N(Input!E57)&gt;0),Input!E57,0)</f>
+        <f>IF(AND(N(Input!D55)=0,N(Input!E55)&gt;0),Input!E55,0)</f>
         <v>0</v>
       </c>
       <c r="F77" s="32"/>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="33" t="str">
-        <f>IF(Input!A58="","",Input!A58)</f>
-        <v>Cliente J</v>
+        <f>IF(Input!A56="","",Input!A56)</f>
+        <v>Cliente H</v>
       </c>
       <c r="B78" s="32"/>
       <c r="C78" s="34" t="s">
         <v>162</v>
       </c>
       <c r="D78" s="35">
-        <f>IF(AND(N(Input!C58)=0,N(Input!D58)&gt;0),Input!D58,0)</f>
-        <v>230</v>
+        <f>IF(AND(N(Input!C56)=0,N(Input!D56)&gt;0),Input!D56,0)</f>
+        <v>0</v>
       </c>
       <c r="E78" s="35">
-        <f>IF(AND(N(Input!D58)=0,N(Input!E58)&gt;0),Input!E58,0)</f>
+        <f>IF(AND(N(Input!D56)=0,N(Input!E56)&gt;0),Input!E56,0)</f>
         <v>0</v>
       </c>
       <c r="F78" s="32"/>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="33" t="str">
-        <f>IF(Input!A59="","",Input!A59)</f>
-        <v/>
+        <f>IF(Input!A57="","",Input!A57)</f>
+        <v>Cliente I</v>
       </c>
       <c r="B79" s="32"/>
       <c r="C79" s="34" t="s">
         <v>162</v>
       </c>
       <c r="D79" s="35">
-        <f>IF(AND(N(Input!C59)=0,N(Input!D59)&gt;0),Input!D59,0)</f>
+        <f>IF(AND(N(Input!C57)=0,N(Input!D57)&gt;0),Input!D57,0)</f>
         <v>0</v>
       </c>
       <c r="E79" s="35">
-        <f>IF(AND(N(Input!D59)=0,N(Input!E59)&gt;0),Input!E59,0)</f>
+        <f>IF(AND(N(Input!D57)=0,N(Input!E57)&gt;0),Input!E57,0)</f>
         <v>0</v>
       </c>
       <c r="F79" s="32"/>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="33" t="str">
-        <f>IF(Input!A60="","",Input!A60)</f>
-        <v/>
+        <f>IF(Input!A58="","",Input!A58)</f>
+        <v>Cliente J</v>
       </c>
       <c r="B80" s="32"/>
       <c r="C80" s="34" t="s">
         <v>162</v>
       </c>
       <c r="D80" s="35">
+        <f>IF(AND(N(Input!C58)=0,N(Input!D58)&gt;0),Input!D58,0)</f>
+        <v>230</v>
+      </c>
+      <c r="E80" s="35">
+        <f>IF(AND(N(Input!D58)=0,N(Input!E58)&gt;0),Input!E58,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F80" s="32"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" s="33" t="str">
+        <f>IF(Input!A59="","",Input!A59)</f>
+        <v/>
+      </c>
+      <c r="B81" s="32"/>
+      <c r="C81" s="34" t="s">
+        <v>162</v>
+      </c>
+      <c r="D81" s="35">
+        <f>IF(AND(N(Input!C59)=0,N(Input!D59)&gt;0),Input!D59,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E81" s="35">
+        <f>IF(AND(N(Input!D59)=0,N(Input!E59)&gt;0),Input!E59,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F81" s="32"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="33" t="str">
+        <f>IF(Input!A60="","",Input!A60)</f>
+        <v/>
+      </c>
+      <c r="B82" s="32"/>
+      <c r="C82" s="34" t="s">
+        <v>162</v>
+      </c>
+      <c r="D82" s="35">
         <f>IF(AND(N(Input!C60)=0,N(Input!D60)&gt;0),Input!D60,0)</f>
         <v>0</v>
       </c>
-      <c r="E80" s="35">
+      <c r="E82" s="35">
         <f>IF(AND(N(Input!D60)=0,N(Input!E60)&gt;0),Input!E60,0)</f>
         <v>0</v>
       </c>
-      <c r="F80" s="32"/>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A81" s="32"/>
-      <c r="B81" s="32"/>
-      <c r="C81" s="32"/>
-      <c r="D81" s="32"/>
-      <c r="E81" s="32"/>
-      <c r="F81" s="32"/>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A82" s="12" t="s">
-        <v>274</v>
-      </c>
-      <c r="B82" s="23"/>
-      <c r="C82" s="23"/>
-      <c r="D82" s="23"/>
-      <c r="E82" s="23"/>
-      <c r="F82" s="23"/>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A83" s="33" t="str">
-        <f>IF(Input!A64="","",Input!A64)</f>
-        <v>Custos legais de um litígio encerrado</v>
-      </c>
+      <c r="F82" s="32"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="32"/>
       <c r="B83" s="32"/>
       <c r="C83" s="32"/>
       <c r="D83" s="32"/>
-      <c r="E83" s="32">
-        <f>IF(AND(N(Input!C64)&lt;&gt;0,N(Input!D64)&lt;&gt;0,N(Input!E64)&lt;&gt;0),1,0)</f>
-        <v>0</v>
-      </c>
+      <c r="E83" s="32"/>
       <c r="F83" s="32"/>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A84" s="33" t="str">
-        <f>IF(Input!A65="","",Input!A65)</f>
-        <v>Certificação ISO 9001 (projeto único)</v>
-      </c>
-      <c r="B84" s="32"/>
-      <c r="C84" s="32"/>
-      <c r="D84" s="32"/>
-      <c r="E84" s="32">
-        <f>IF(AND(N(Input!C65)&lt;&gt;0,N(Input!D65)&lt;&gt;0,N(Input!E65)&lt;&gt;0),1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F84" s="32"/>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="B84" s="23"/>
+      <c r="C84" s="23"/>
+      <c r="D84" s="23"/>
+      <c r="E84" s="23"/>
+      <c r="F84" s="23"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="33" t="str">
-        <f>IF(Input!A66="","",Input!A66)</f>
-        <v>Migração do sistema informático (ERP)</v>
+        <f>IF(Input!A64="","",Input!A64)</f>
+        <v>Custos legais de um litígio encerrado</v>
       </c>
       <c r="B85" s="32"/>
       <c r="C85" s="32"/>
       <c r="D85" s="32"/>
       <c r="E85" s="32">
-        <f>IF(AND(N(Input!C66)&lt;&gt;0,N(Input!D66)&lt;&gt;0,N(Input!E66)&lt;&gt;0),1,0)</f>
+        <f>IF(AND(N(Input!C64)&lt;&gt;0,N(Input!D64)&lt;&gt;0,N(Input!E64)&lt;&gt;0),1,0)</f>
         <v>0</v>
       </c>
       <c r="F85" s="32"/>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="33" t="str">
-        <f>IF(Input!A67="","",Input!A67)</f>
-        <v/>
+        <f>IF(Input!A65="","",Input!A65)</f>
+        <v>Certificação ISO 9001 (projeto único)</v>
       </c>
       <c r="B86" s="32"/>
       <c r="C86" s="32"/>
       <c r="D86" s="32"/>
       <c r="E86" s="32">
-        <f>IF(AND(N(Input!C67)&lt;&gt;0,N(Input!D67)&lt;&gt;0,N(Input!E67)&lt;&gt;0),1,0)</f>
+        <f>IF(AND(N(Input!C65)&lt;&gt;0,N(Input!D65)&lt;&gt;0,N(Input!E65)&lt;&gt;0),1,0)</f>
         <v>0</v>
       </c>
       <c r="F86" s="32"/>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="33" t="str">
-        <f>IF(Input!A68="","",Input!A68)</f>
-        <v/>
+        <f>IF(Input!A66="","",Input!A66)</f>
+        <v>Migração do sistema informático (ERP)</v>
       </c>
       <c r="B87" s="32"/>
       <c r="C87" s="32"/>
       <c r="D87" s="32"/>
       <c r="E87" s="32">
-        <f>IF(AND(N(Input!C68)&lt;&gt;0,N(Input!D68)&lt;&gt;0,N(Input!E68)&lt;&gt;0),1,0)</f>
+        <f>IF(AND(N(Input!C66)&lt;&gt;0,N(Input!D66)&lt;&gt;0,N(Input!E66)&lt;&gt;0),1,0)</f>
         <v>0</v>
       </c>
       <c r="F87" s="32"/>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A88" s="32"/>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" s="33" t="str">
+        <f>IF(Input!A67="","",Input!A67)</f>
+        <v/>
+      </c>
       <c r="B88" s="32"/>
       <c r="C88" s="32"/>
       <c r="D88" s="32"/>
-      <c r="E88" s="32"/>
+      <c r="E88" s="32">
+        <f>IF(AND(N(Input!C67)&lt;&gt;0,N(Input!D67)&lt;&gt;0,N(Input!E67)&lt;&gt;0),1,0)</f>
+        <v>0</v>
+      </c>
       <c r="F88" s="32"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" s="33" t="str">
+        <f>IF(Input!A68="","",Input!A68)</f>
+        <v/>
+      </c>
+      <c r="B89" s="32"/>
+      <c r="C89" s="32"/>
+      <c r="D89" s="32"/>
+      <c r="E89" s="32">
+        <f>IF(AND(N(Input!C68)&lt;&gt;0,N(Input!D68)&lt;&gt;0,N(Input!E68)&lt;&gt;0),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F89" s="32"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" s="32"/>
+      <c r="B90" s="32"/>
+      <c r="C90" s="32"/>
+      <c r="D90" s="32"/>
+      <c r="E90" s="32"/>
+      <c r="F90" s="32"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5899,7 +5953,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:V24"/>
-  <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -5919,17 +5973,17 @@
     <col min="21" max="22" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="17.600000000000001" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:22" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>277</v>
       </c>
@@ -5997,7 +6051,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="5" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>293</v>
       </c>
@@ -6076,7 +6130,7 @@
         <v>R01 · Maior cliente acima do limite (limite: 20%)</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>301</v>
       </c>
@@ -6155,7 +6209,7 @@
         <v>R02 · Cliente novo com peso relevante nas vendas (limite: 5%)</v>
       </c>
     </row>
-    <row r="7" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>308</v>
       </c>
@@ -6234,7 +6288,7 @@
         <v>R03 · Variação forte da margem bruta (limite: 3 p.p.)</v>
       </c>
     </row>
-    <row r="8" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>317</v>
       </c>
@@ -6245,25 +6299,25 @@
         <v>319</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>190</v>
+        <v>443</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>295</v>
       </c>
       <c r="F8" s="36">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="G8" s="37">
-        <f>Métricas!C21</f>
-        <v>3.9473684210526317E-3</v>
+        <f>Métricas!C22</f>
+        <v>4.5592705167173252E-2</v>
       </c>
       <c r="H8" s="37">
-        <f>Métricas!D21</f>
-        <v>3.459119496855346E-3</v>
+        <f>Métricas!D22</f>
+        <v>3.8194444444444448E-2</v>
       </c>
       <c r="I8" s="37">
-        <f>Métricas!E21</f>
-        <v>3.8922155688622755E-3</v>
+        <f>Métricas!E22</f>
+        <v>4.4858523119392688E-2</v>
       </c>
       <c r="J8" s="9" t="str">
         <f t="shared" ref="J8:L13" si="3">IF(ISNUMBER(G8),IF(G8&gt;$F8,"Sim","Não"),"n.d.")</f>
@@ -6285,16 +6339,17 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="O8" s="11" t="s">
-        <v>296</v>
+      <c r="O8" s="11" t="str">
+        <f>IF(MAX(G8:I8)&gt;0.25,"Alta","Média")</f>
+        <v>Média</v>
       </c>
       <c r="P8" s="10" t="str">
         <f>IF(M8="Sim",COUNTIF(M$5:M8,"Sim"),"")</f>
         <v/>
       </c>
       <c r="Q8" s="10" t="str">
-        <f>IFERROR("Outros rendimentos — 2023: "&amp;ROUND(Input!C11,0)&amp;"; 2024: "&amp;ROUND(Input!D11,0)&amp;"; 2025: "&amp;ROUND(Input!E11,0)&amp;" ("&amp;ROUND(Métricas!E21*100,1)&amp;"%"&amp;" das vendas; variação de "&amp;ROUND(Métricas!E22*100,1)&amp;"%"&amp;"). Fonte: "&amp;Input!$F$11,"Ver folha Métricas")</f>
-        <v>Outros rendimentos — 2023: 60; 2024: 55; 2025: 65 (0,4% das vendas; variação de 18,2%). Fonte: DRE!B11:D11</v>
+        <f>IFERROR("Outros rendimentos — 2023: "&amp;ROUND(Input!C11,0)&amp;"; 2024: "&amp;ROUND(Input!D11,0)&amp;"; 2025: "&amp;ROUND(Input!E11,0)&amp;" ("&amp;ROUND(Métricas!E22*100,1)&amp;"% do EBITDA e "&amp;ROUND(Métricas!E21*100,1)&amp;"% das vendas em 2025; variação de "&amp;ROUND(Métricas!E23*100,1)&amp;"%"&amp;"). Fonte: "&amp;Input!$F$11,"Ver folha Métricas")</f>
+        <v>Outros rendimentos — 2023: 60; 2024: 55; 2025: 65 (4,5% do EBITDA e 0,4% das vendas em 2025; variação de 18,2%). Fonte: DRE!B11:D11</v>
       </c>
       <c r="R8" s="10" t="s">
         <v>320</v>
@@ -6309,11 +6364,11 @@
         <v>323</v>
       </c>
       <c r="V8" s="10" t="str">
-        <f>"R04"&amp;" · "&amp;C8&amp;" (limite: "&amp;ROUND(F8*100,0)&amp;"%"&amp;")"</f>
-        <v>R04 · Outros rendimentos relevantes dentro do EBITDA (limite: 1%)</v>
-      </c>
-    </row>
-    <row r="9" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+        <f>"R04"&amp;" · "&amp;C8&amp;" (limite: "&amp;ROUND(F8*100,0)&amp;"%"&amp;"; Alta acima de 25%)"</f>
+        <v>R04 · Outros rendimentos relevantes dentro do EBITDA (limite: 10%; Alta acima de 25%)</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>324</v>
       </c>
@@ -6333,15 +6388,15 @@
         <v>0.1</v>
       </c>
       <c r="G9" s="37">
-        <f>Métricas!C28</f>
+        <f>Métricas!C29</f>
         <v>1.8996960486322188E-2</v>
       </c>
       <c r="H9" s="37">
-        <f>Métricas!D28</f>
+        <f>Métricas!D29</f>
         <v>2.4305555555555556E-2</v>
       </c>
       <c r="I9" s="37">
-        <f>Métricas!E28</f>
+        <f>Métricas!E29</f>
         <v>2.7605244996549344E-2</v>
       </c>
       <c r="J9" s="9" t="str">
@@ -6372,7 +6427,7 @@
         <v/>
       </c>
       <c r="Q9" s="10" t="str">
-        <f>IFERROR("Ajustes em % do EBITDA reportado — "&amp;"2023: "&amp;ROUND(Métricas!C28*100,1)&amp;"%"&amp;"; 2024: "&amp;ROUND(Métricas!D28*100,1)&amp;"%"&amp;"; 2025: "&amp;ROUND(Métricas!E28*100,1)&amp;"%"&amp;". EBITDA 2025: reportado "&amp;ROUND(Métricas!E19,0)&amp;", ajustado pela gestão "&amp;ROUND(Métricas!E27,0)&amp;". Fonte: "&amp;Input!$F$64&amp;" e seguintes; "&amp;Input!$F$6,"Ver folha Métricas")</f>
+        <f>IFERROR("Ajustes em % do EBITDA reportado — "&amp;"2023: "&amp;ROUND(Métricas!C29*100,1)&amp;"%"&amp;"; 2024: "&amp;ROUND(Métricas!D29*100,1)&amp;"%"&amp;"; 2025: "&amp;ROUND(Métricas!E29*100,1)&amp;"%"&amp;". EBITDA 2025: reportado "&amp;ROUND(Métricas!E19,0)&amp;", ajustado pela gestão "&amp;ROUND(Métricas!E28,0)&amp;". Fonte: "&amp;Input!$F$64&amp;" e seguintes; "&amp;Input!$F$6,"Ver folha Métricas")</f>
         <v>Ajustes em % do EBITDA reportado — 2023: 1,9%; 2024: 2,4%; 2025: 2,8%. EBITDA 2025: reportado 1449, ajustado pela gestão 1489. Fonte: EBITDA Ajustado!B8:D8 e seguintes; DRE!B5:D5</v>
       </c>
       <c r="R9" s="10" t="s">
@@ -6392,7 +6447,7 @@
         <v>R05 · Ajustes da gestão elevados (limite: 10%)</v>
       </c>
     </row>
-    <row r="10" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>330</v>
       </c>
@@ -6412,15 +6467,15 @@
         <v>0</v>
       </c>
       <c r="G10" s="41" t="str">
-        <f>Métricas!C29</f>
+        <f>Métricas!C30</f>
         <v>n.d.</v>
       </c>
       <c r="H10" s="41" t="str">
-        <f>Métricas!D29</f>
+        <f>Métricas!D30</f>
         <v>n.d.</v>
       </c>
       <c r="I10" s="41">
-        <f>Métricas!E29</f>
+        <f>Métricas!E30</f>
         <v>0</v>
       </c>
       <c r="J10" s="9" t="str">
@@ -6451,7 +6506,7 @@
         <v/>
       </c>
       <c r="Q10" s="10" t="str">
-        <f>IFERROR(ROUND(Métricas!E29,0)&amp;" ajuste(s) aparece(m) em 2023, 2024 e 2025 (ex.: "&amp;Métricas!E30&amp;"). Fonte: "&amp;Input!$F$64&amp;" e seguintes","Ver folha Métricas")</f>
+        <f>IFERROR(ROUND(Métricas!E30,0)&amp;" ajuste(s) aparece(m) em 2023, 2024 e 2025 (ex.: "&amp;Métricas!E31&amp;"). Fonte: "&amp;Input!$F$64&amp;" e seguintes","Ver folha Métricas")</f>
         <v>0 ajuste(s) aparece(m) em 2023, 2024 e 2025 (ex.: —). Fonte: EBITDA Ajustado!B8:D8 e seguintes</v>
       </c>
       <c r="R10" s="10" t="s">
@@ -6471,7 +6526,7 @@
         <v>R06 · Ajuste 'não recorrente' que se repete todos os anos (limite: mais de 0)</v>
       </c>
     </row>
-    <row r="11" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>338</v>
       </c>
@@ -6491,15 +6546,15 @@
         <v>10</v>
       </c>
       <c r="G11" s="39" t="str">
-        <f>Métricas!C33</f>
+        <f>Métricas!C34</f>
         <v>n.d.</v>
       </c>
       <c r="H11" s="39">
-        <f>Métricas!D33</f>
+        <f>Métricas!D34</f>
         <v>-3.5162460760740366E-2</v>
       </c>
       <c r="I11" s="39">
-        <f>Métricas!E33</f>
+        <f>Métricas!E34</f>
         <v>0.15373864430467954</v>
       </c>
       <c r="J11" s="9" t="str">
@@ -6530,7 +6585,7 @@
         <v/>
       </c>
       <c r="Q11" s="10" t="str">
-        <f>IFERROR("Clientes +"&amp;ROUND(Métricas!E32*100,1)&amp;"%"&amp;" vs. vendas +"&amp;ROUND(Métricas!E7*100,1)&amp;"%"&amp;" em 2025 (diferença de "&amp;ROUND(Métricas!E33,1)&amp;" p.p.; 2024: "&amp;ROUND(Métricas!D33,1)&amp;" p.p.). DSO: "&amp;ROUND(Métricas!D34,1)&amp;" → "&amp;ROUND(Métricas!E34,1)&amp;" dias. Fonte: "&amp;Input!$F$22&amp;"; "&amp;Input!$F$6,"Ver folha Métricas")</f>
+        <f>IFERROR("Clientes +"&amp;ROUND(Métricas!E33*100,1)&amp;"%"&amp;" vs. vendas +"&amp;ROUND(Métricas!E7*100,1)&amp;"%"&amp;" em 2025 (diferença de "&amp;ROUND(Métricas!E34,1)&amp;" p.p.; 2024: "&amp;ROUND(Métricas!D34,1)&amp;" p.p.). DSO: "&amp;ROUND(Métricas!D35,1)&amp;" → "&amp;ROUND(Métricas!E35,1)&amp;" dias. Fonte: "&amp;Input!$F$22&amp;"; "&amp;Input!$F$6,"Ver folha Métricas")</f>
         <v>Clientes +5,2% vs. vendas +5% em 2025 (diferença de 0,2 p.p.; 2024: 0 p.p.). DSO: 62 → 62,1 dias. Fonte: Balanço!B9:E9; DRE!B5:D5</v>
       </c>
       <c r="R11" s="10" t="s">
@@ -6550,7 +6605,7 @@
         <v>R07 · Contas a receber crescem acima das vendas (limite: 10 p.p.)</v>
       </c>
     </row>
-    <row r="12" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>345</v>
       </c>
@@ -6570,15 +6625,15 @@
         <v>15</v>
       </c>
       <c r="G12" s="43" t="str">
-        <f>Métricas!C35</f>
+        <f>Métricas!C36</f>
         <v>n.d.</v>
       </c>
       <c r="H12" s="43">
-        <f>Métricas!D35</f>
+        <f>Métricas!D36</f>
         <v>-2.0841608738834339E-2</v>
       </c>
       <c r="I12" s="43">
-        <f>Métricas!E35</f>
+        <f>Métricas!E36</f>
         <v>9.0724211953457257E-2</v>
       </c>
       <c r="J12" s="9" t="str">
@@ -6609,7 +6664,7 @@
         <v/>
       </c>
       <c r="Q12" s="10" t="str">
-        <f>IFERROR("DSO — "&amp;"2023: "&amp;ROUND(Métricas!C34,1)&amp;"; 2024: "&amp;ROUND(Métricas!D34,1)&amp;"; 2025: "&amp;ROUND(Métricas!E34,1)&amp;" dias. Fonte: "&amp;Input!$F$22&amp;"; "&amp;Input!$F$6,"Ver folha Métricas")</f>
+        <f>IFERROR("DSO — "&amp;"2023: "&amp;ROUND(Métricas!C35,1)&amp;"; 2024: "&amp;ROUND(Métricas!D35,1)&amp;"; 2025: "&amp;ROUND(Métricas!E35,1)&amp;" dias. Fonte: "&amp;Input!$F$22&amp;"; "&amp;Input!$F$6,"Ver folha Métricas")</f>
         <v>DSO — 2023: 62; 2024: 62; 2025: 62,1 dias. Fonte: Balanço!B9:E9; DRE!B5:D5</v>
       </c>
       <c r="R12" s="10" t="s">
@@ -6629,7 +6684,7 @@
         <v>R08 · Aumento forte do prazo de recebimento (limite: 15 dias)</v>
       </c>
     </row>
-    <row r="13" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>352</v>
       </c>
@@ -6649,15 +6704,15 @@
         <v>10</v>
       </c>
       <c r="G13" s="39" t="str">
-        <f>Métricas!C38</f>
+        <f>Métricas!C39</f>
         <v>n.d.</v>
       </c>
       <c r="H13" s="39">
-        <f>Métricas!D38</f>
+        <f>Métricas!D39</f>
         <v>-2.960526315789469E-2</v>
       </c>
       <c r="I13" s="39">
-        <f>Métricas!E38</f>
+        <f>Métricas!E39</f>
         <v>-0.20641194554238407</v>
       </c>
       <c r="J13" s="9" t="str">
@@ -6688,7 +6743,7 @@
         <v/>
       </c>
       <c r="Q13" s="10" t="str">
-        <f>IFERROR("Inventários +"&amp;ROUND(Métricas!E36*100,1)&amp;"%"&amp;" vs. CMV +"&amp;ROUND(Métricas!E37*100,1)&amp;"%"&amp;" em 2025 (diferença de "&amp;ROUND(Métricas!E38,1)&amp;" p.p.). DIO: "&amp;ROUND(Métricas!D39,1)&amp;" → "&amp;ROUND(Métricas!E39,1)&amp;" dias. Fonte: "&amp;Input!$F$21&amp;"; "&amp;Input!$F$7,"Ver folha Métricas")</f>
+        <f>IFERROR("Inventários +"&amp;ROUND(Métricas!E37*100,1)&amp;"%"&amp;" vs. CMV +"&amp;ROUND(Métricas!E38*100,1)&amp;"%"&amp;" em 2025 (diferença de "&amp;ROUND(Métricas!E39,1)&amp;" p.p.). DIO: "&amp;ROUND(Métricas!D40,1)&amp;" → "&amp;ROUND(Métricas!E40,1)&amp;" dias. Fonte: "&amp;Input!$F$21&amp;"; "&amp;Input!$F$7,"Ver folha Métricas")</f>
         <v>Inventários +5,6% vs. CMV +5,8% em 2025 (diferença de -0,2 p.p.). DIO: 75 → 74,9 dias. Fonte: Balanço!B8:E8; DRE!B6:D6</v>
       </c>
       <c r="R13" s="10" t="s">
@@ -6708,7 +6763,7 @@
         <v>R09 · Inventários crescem acima do CMV (limite: 10 p.p.)</v>
       </c>
     </row>
-    <row r="14" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>359</v>
       </c>
@@ -6728,15 +6783,15 @@
         <v>0.7</v>
       </c>
       <c r="G14" s="37">
-        <f>Métricas!C44</f>
+        <f>Métricas!C45</f>
         <v>0.90729483282674772</v>
       </c>
       <c r="H14" s="37">
-        <f>Métricas!D44</f>
+        <f>Métricas!D45</f>
         <v>0.91111111111111109</v>
       </c>
       <c r="I14" s="37">
-        <f>Métricas!E44</f>
+        <f>Métricas!E45</f>
         <v>0.89302967563837132</v>
       </c>
       <c r="J14" s="9" t="str">
@@ -6759,16 +6814,17 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="O14" s="11" t="s">
-        <v>296</v>
+      <c r="O14" s="11" t="str">
+        <f>IF(ISNUMBER(Métricas!E46),IF(Métricas!E46&lt;F14,"Alta","Média"),"Média")</f>
+        <v>Média</v>
       </c>
       <c r="P14" s="10" t="str">
         <f>IF(M14="Sim",COUNTIF(M$5:M14,"Sim"),"")</f>
         <v/>
       </c>
       <c r="Q14" s="10" t="str">
-        <f>IFERROR("Conversão de caixa — "&amp;"2023: "&amp;ROUND(Métricas!C44*100,1)&amp;"%"&amp;"; 2024: "&amp;ROUND(Métricas!D44*100,1)&amp;"%"&amp;"; 2025: "&amp;ROUND(Métricas!E44*100,1)&amp;"%"&amp;". FCO 2025: "&amp;ROUND(Métricas!E45,0)&amp;". Fonte: "&amp;Input!$F$40&amp;"; "&amp;Input!$F$6,"Ver folha Métricas")</f>
-        <v>Conversão de caixa — 2023: 90,7%; 2024: 91,1%; 2025: 89,3%. FCO 2025: 985. Fonte: DFC!B15:D15; DRE!B5:D5</v>
+        <f>IFERROR("Conversão de caixa — 2023: "&amp;ROUND(Métricas!C45*100,1)&amp;"%; 2024: "&amp;ROUND(Métricas!D45*100,1)&amp;"%; 2025: "&amp;ROUND(Métricas!E45*100,1)&amp;"%; os anos analisados juntos: "&amp;ROUND(Métricas!E46*100,1)&amp;"%. FCO 2025: "&amp;ROUND(Métricas!E47,0)&amp;". Fonte: "&amp;Input!$F$40&amp;"; "&amp;Input!$F$6,"Ver folha Métricas")</f>
+        <v>Conversão de caixa — 2023: 90,7%; 2024: 91,1%; 2025: 89,3%; os anos analisados juntos: 90,4%. FCO 2025: 985. Fonte: DFC!B15:D15; DRE!B5:D5</v>
       </c>
       <c r="R14" s="10" t="s">
         <v>362</v>
@@ -6783,11 +6839,11 @@
         <v>365</v>
       </c>
       <c r="V14" s="10" t="str">
-        <f>"R10"&amp;" · "&amp;C14&amp;" (limite: "&amp;ROUND(F14*100,0)&amp;"%"&amp;")"</f>
-        <v>R10 · Fraca conversão do EBITDA em caixa (limite: 70%)</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+        <f>"R10"&amp;" · "&amp;C14&amp;" (limite: "&amp;ROUND(F14*100,0)&amp;"%"&amp;"; Alta quando os anos analisados, juntos, ficam abaixo)"</f>
+        <v>R10 · Fraca conversão do EBITDA em caixa (limite: 70%; Alta quando os anos analisados, juntos, ficam abaixo)</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>366</v>
       </c>
@@ -6807,15 +6863,15 @@
         <v>0.4</v>
       </c>
       <c r="G15" s="37">
-        <f>Métricas!C50</f>
+        <f>Métricas!C52</f>
         <v>0.17647058823529413</v>
       </c>
       <c r="H15" s="37">
-        <f>Métricas!D50</f>
+        <f>Métricas!D52</f>
         <v>0.21428571428571427</v>
       </c>
       <c r="I15" s="37">
-        <f>Métricas!E50</f>
+        <f>Métricas!E52</f>
         <v>0.27272727272727271</v>
       </c>
       <c r="J15" s="9" t="str">
@@ -6846,7 +6902,7 @@
         <v/>
       </c>
       <c r="Q15" s="10" t="str">
-        <f>IFERROR("Dívida a vencer em 12 meses — "&amp;"2023: "&amp;ROUND(Métricas!C50*100,1)&amp;"%"&amp;"; 2024: "&amp;ROUND(Métricas!D50*100,1)&amp;"%"&amp;"; 2025: "&amp;ROUND(Métricas!E50*100,1)&amp;"%"&amp;" ("&amp;ROUND(Input!E30,0)&amp;" de "&amp;ROUND(Métricas!E49,0)&amp;" em 2025). Fonte: "&amp;Input!$F$30&amp;"; "&amp;Input!$F$27,"Ver folha Métricas")</f>
+        <f>IFERROR("Dívida a vencer em 12 meses — "&amp;"2023: "&amp;ROUND(Métricas!C52*100,1)&amp;"%"&amp;"; 2024: "&amp;ROUND(Métricas!D52*100,1)&amp;"%"&amp;"; 2025: "&amp;ROUND(Métricas!E52*100,1)&amp;"%"&amp;" ("&amp;ROUND(Input!E30,0)&amp;" de "&amp;ROUND(Métricas!E51,0)&amp;" em 2025). Fonte: "&amp;Input!$F$30&amp;"; "&amp;Input!$F$27,"Ver folha Métricas")</f>
         <v>Dívida a vencer em 12 meses — 2023: 17,6%; 2024: 21,4%; 2025: 27,3% (360 de 1320 em 2025). Fonte: Balanço!B23:E23; Balanço!B20:E20</v>
       </c>
       <c r="R15" s="10" t="s">
@@ -6866,7 +6922,7 @@
         <v>R11 · Dívida concentrada nos próximos 12 meses (limite: 40%)</v>
       </c>
     </row>
-    <row r="16" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>372</v>
       </c>
@@ -6886,15 +6942,15 @@
         <v>1</v>
       </c>
       <c r="G16" s="45">
-        <f>Métricas!C58</f>
+        <f>Métricas!C60</f>
         <v>0</v>
       </c>
       <c r="H16" s="45">
-        <f>Métricas!D58</f>
+        <f>Métricas!D60</f>
         <v>0</v>
       </c>
       <c r="I16" s="45">
-        <f>Métricas!E58</f>
+        <f>Métricas!E60</f>
         <v>0</v>
       </c>
       <c r="J16" s="9" t="str">
@@ -6925,7 +6981,7 @@
         <v/>
       </c>
       <c r="Q16" s="10" t="str">
-        <f>IFERROR("Diferença no balanço — "&amp;"2023: "&amp;ROUND(Métricas!C58,0)&amp;"; 2024: "&amp;ROUND(Métricas!D58,0)&amp;"; 2025: "&amp;ROUND(Métricas!E58,0)&amp;". Fonte: Input, secção Balanço","Ver folha Métricas")</f>
+        <f>IFERROR("Diferença no balanço — "&amp;"2023: "&amp;ROUND(Métricas!C60,0)&amp;"; 2024: "&amp;ROUND(Métricas!D60,0)&amp;"; 2025: "&amp;ROUND(Métricas!E60,0)&amp;". Fonte: Input, secção Balanço","Ver folha Métricas")</f>
         <v>Diferença no balanço — 2023: 0; 2024: 0; 2025: 0. Fonte: Input, secção Balanço</v>
       </c>
       <c r="R16" s="10" t="s">
@@ -6945,7 +7001,7 @@
         <v>R12 · Balanço não fecha (limite: 1 mil €)</v>
       </c>
     </row>
-    <row r="17" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>379</v>
       </c>
@@ -6965,15 +7021,15 @@
         <v>1</v>
       </c>
       <c r="G17" s="45">
-        <f>Métricas!C59</f>
+        <f>Métricas!C61</f>
         <v>0</v>
       </c>
       <c r="H17" s="45">
-        <f>Métricas!D59</f>
+        <f>Métricas!D61</f>
         <v>0</v>
       </c>
       <c r="I17" s="45">
-        <f>Métricas!E59</f>
+        <f>Métricas!E61</f>
         <v>0</v>
       </c>
       <c r="J17" s="9" t="str">
@@ -7004,7 +7060,7 @@
         <v/>
       </c>
       <c r="Q17" s="10" t="str">
-        <f>IFERROR("Caixa final da DFC − caixa do balanço — "&amp;"2023: "&amp;ROUND(Métricas!C59,0)&amp;"; 2024: "&amp;ROUND(Métricas!D59,0)&amp;"; 2025: "&amp;ROUND(Métricas!E59,0)&amp;". Fonte: "&amp;Input!$F$46&amp;"; "&amp;Input!$F$24,"Ver folha Métricas")</f>
+        <f>IFERROR("Caixa final da DFC − caixa do balanço — "&amp;"2023: "&amp;ROUND(Métricas!C61,0)&amp;"; 2024: "&amp;ROUND(Métricas!D61,0)&amp;"; 2025: "&amp;ROUND(Métricas!E61,0)&amp;". Fonte: "&amp;Input!$F$46&amp;"; "&amp;Input!$F$24,"Ver folha Métricas")</f>
         <v>Caixa final da DFC − caixa do balanço — 2023: 0; 2024: 0; 2025: 0. Fonte: DFC!B31:D31; Balanço!B11:E11</v>
       </c>
       <c r="R17" s="10" t="s">
@@ -7024,7 +7080,7 @@
         <v>R13 · Caixa da DFC não bate com o balanço (limite: 1 mil €)</v>
       </c>
     </row>
-    <row r="18" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
         <v>385</v>
       </c>
@@ -7044,15 +7100,15 @@
         <v>1</v>
       </c>
       <c r="G18" s="45">
-        <f>Métricas!C60</f>
+        <f>Métricas!C62</f>
         <v>0</v>
       </c>
       <c r="H18" s="45">
-        <f>Métricas!D60</f>
+        <f>Métricas!D62</f>
         <v>0</v>
       </c>
       <c r="I18" s="45">
-        <f>Métricas!E60</f>
+        <f>Métricas!E62</f>
         <v>0</v>
       </c>
       <c r="J18" s="9" t="str">
@@ -7083,7 +7139,7 @@
         <v/>
       </c>
       <c r="Q18" s="10" t="str">
-        <f>IFERROR("Diferença entre DFC e balanço nas variações de capital de giro — "&amp;"2023: "&amp;ROUND(Métricas!C60,0)&amp;"; 2024: "&amp;ROUND(Métricas!D60,0)&amp;"; 2025: "&amp;ROUND(Métricas!E60,0)&amp;". Fonte: "&amp;Input!$F$35&amp;" a "&amp;Input!$F$39,"Ver folha Métricas")</f>
+        <f>IFERROR("Diferença entre DFC e balanço nas variações de capital de giro — "&amp;"2023: "&amp;ROUND(Métricas!C62,0)&amp;"; 2024: "&amp;ROUND(Métricas!D62,0)&amp;"; 2025: "&amp;ROUND(Métricas!E62,0)&amp;". Fonte: "&amp;Input!$F$35&amp;" a "&amp;Input!$F$39,"Ver folha Métricas")</f>
         <v>Diferença entre DFC e balanço nas variações de capital de giro — 2023: 0; 2024: 0; 2025: 0. Fonte: DFC!B10:D10 a DFC!B14:D14</v>
       </c>
       <c r="R18" s="10" t="s">
@@ -7103,7 +7159,7 @@
         <v>R14 · Variações de capital de giro da DFC não batem com o balanço (limite: 1 mil €)</v>
       </c>
     </row>
-    <row r="19" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
         <v>392</v>
       </c>
@@ -7123,15 +7179,15 @@
         <v>1</v>
       </c>
       <c r="G19" s="45">
-        <f>Métricas!C61</f>
+        <f>Métricas!C63</f>
         <v>0</v>
       </c>
       <c r="H19" s="45">
-        <f>Métricas!D61</f>
+        <f>Métricas!D63</f>
         <v>0</v>
       </c>
       <c r="I19" s="45">
-        <f>Métricas!E61</f>
+        <f>Métricas!E63</f>
         <v>0</v>
       </c>
       <c r="J19" s="9" t="str">
@@ -7162,7 +7218,7 @@
         <v/>
       </c>
       <c r="Q19" s="10" t="str">
-        <f>IFERROR("Diferença no resultado líquido — "&amp;"2023: "&amp;ROUND(Métricas!C61,0)&amp;"; 2024: "&amp;ROUND(Métricas!D61,0)&amp;"; 2025: "&amp;ROUND(Métricas!E61,0)&amp;". Fonte: "&amp;Input!$F$16&amp;"; "&amp;Input!$F$26&amp;"; "&amp;Input!$F$34,"Ver folha Métricas")</f>
+        <f>IFERROR("Diferença no resultado líquido — "&amp;"2023: "&amp;ROUND(Métricas!C63,0)&amp;"; 2024: "&amp;ROUND(Métricas!D63,0)&amp;"; 2025: "&amp;ROUND(Métricas!E63,0)&amp;". Fonte: "&amp;Input!$F$16&amp;"; "&amp;Input!$F$26&amp;"; "&amp;Input!$F$34,"Ver folha Métricas")</f>
         <v>Diferença no resultado líquido — 2023: 0; 2024: 0; 2025: 0. Fonte: DRE!B19:D19; Balanço!B18:E18; DFC!B5:D5</v>
       </c>
       <c r="R19" s="10" t="s">
@@ -7182,7 +7238,7 @@
         <v>R15 · Resultado líquido diferente entre demonstrações (limite: 1 mil €)</v>
       </c>
     </row>
-    <row r="20" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
         <v>399</v>
       </c>
@@ -7202,15 +7258,15 @@
         <v>1</v>
       </c>
       <c r="G20" s="45">
-        <f>Métricas!C62</f>
+        <f>Métricas!C64</f>
         <v>0</v>
       </c>
       <c r="H20" s="45">
-        <f>Métricas!D62</f>
+        <f>Métricas!D64</f>
         <v>0</v>
       </c>
       <c r="I20" s="45">
-        <f>Métricas!E62</f>
+        <f>Métricas!E64</f>
         <v>0</v>
       </c>
       <c r="J20" s="9" t="str">
@@ -7241,7 +7297,7 @@
         <v/>
       </c>
       <c r="Q20" s="10" t="str">
-        <f>IFERROR("Vendas por cliente − vendas da DRE — "&amp;"2023: "&amp;ROUND(Métricas!C62,0)&amp;"; 2024: "&amp;ROUND(Métricas!D62,0)&amp;"; 2025: "&amp;ROUND(Métricas!E62,0)&amp;". Fonte: Input, secção Vendas por cliente","Ver folha Métricas")</f>
+        <f>IFERROR("Vendas por cliente − vendas da DRE — "&amp;"2023: "&amp;ROUND(Métricas!C64,0)&amp;"; 2024: "&amp;ROUND(Métricas!D64,0)&amp;"; 2025: "&amp;ROUND(Métricas!E64,0)&amp;". Fonte: Input, secção Vendas por cliente","Ver folha Métricas")</f>
         <v>Vendas por cliente − vendas da DRE — 2023: 0; 2024: 0; 2025: 0. Fonte: Input, secção Vendas por cliente</v>
       </c>
       <c r="R20" s="10" t="s">
@@ -7261,7 +7317,7 @@
         <v>R16 · Vendas por cliente não somam as vendas da DRE (limite: 1 mil €)</v>
       </c>
     </row>
-    <row r="21" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
         <v>406</v>
       </c>
@@ -7281,15 +7337,15 @@
         <v>1</v>
       </c>
       <c r="G21" s="45" t="str">
-        <f>Métricas!C63</f>
+        <f>Métricas!C65</f>
         <v>n.d.</v>
       </c>
       <c r="H21" s="45" t="str">
-        <f>Métricas!D63</f>
+        <f>Métricas!D65</f>
         <v>n.d.</v>
       </c>
       <c r="I21" s="45">
-        <f>Métricas!E63</f>
+        <f>Métricas!E65</f>
         <v>0</v>
       </c>
       <c r="J21" s="9" t="str">
@@ -7320,7 +7376,7 @@
         <v/>
       </c>
       <c r="Q21" s="10" t="str">
-        <f>IFERROR("Mapa da dívida − balanço em 2025: "&amp;ROUND(Métricas!E63,0)&amp;". Fonte: "&amp;Input!$F$71&amp;"; "&amp;Input!$F$30,"Ver folha Métricas")</f>
+        <f>IFERROR("Mapa da dívida − balanço em 2025: "&amp;ROUND(Métricas!E65,0)&amp;". Fonte: "&amp;Input!$F$71&amp;"; "&amp;Input!$F$30,"Ver folha Métricas")</f>
         <v>Mapa da dívida − balanço em 2025: 0. Fonte: Dívida!D7; Balanço!B23:E23</v>
       </c>
       <c r="R21" s="10" t="s">
@@ -7340,7 +7396,7 @@
         <v>R17 · Mapa da dívida não bate com o balanço (limite: 1 mil €)</v>
       </c>
     </row>
-    <row r="22" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
         <v>413</v>
       </c>
@@ -7360,15 +7416,15 @@
         <v>0</v>
       </c>
       <c r="G22" s="41" t="str">
-        <f>Métricas!C65</f>
+        <f>Métricas!C67</f>
         <v>n.d.</v>
       </c>
       <c r="H22" s="41" t="str">
-        <f>Métricas!D65</f>
+        <f>Métricas!D67</f>
         <v>n.d.</v>
       </c>
       <c r="I22" s="41">
-        <f>Métricas!E65</f>
+        <f>Métricas!E67</f>
         <v>0</v>
       </c>
       <c r="J22" s="9" t="str">
@@ -7399,7 +7455,7 @@
         <v/>
       </c>
       <c r="Q22" s="10" t="str">
-        <f>IFERROR(ROUND(Métricas!E65,0)&amp;" documento(s) em falta: "&amp;Métricas!E66&amp;". Fonte: Input, Documentos recebidos","Ver folha Métricas")</f>
+        <f>IFERROR(ROUND(Métricas!E67,0)&amp;" documento(s) em falta: "&amp;Métricas!E68&amp;". Fonte: Input, Documentos recebidos","Ver folha Métricas")</f>
         <v>0 documento(s) em falta: —. Fonte: Input, Documentos recebidos</v>
       </c>
       <c r="R22" s="10" t="s">
@@ -7419,7 +7475,7 @@
         <v>R18 · Documentos obrigatórios em falta (limite: mais de 0)</v>
       </c>
     </row>
-    <row r="23" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
         <v>419</v>
       </c>
@@ -7439,15 +7495,15 @@
         <v>0.05</v>
       </c>
       <c r="G23" s="37">
-        <f>Métricas!C24</f>
+        <f>Métricas!C25</f>
         <v>0</v>
       </c>
       <c r="H23" s="37">
-        <f>Métricas!D24</f>
+        <f>Métricas!D25</f>
         <v>0</v>
       </c>
       <c r="I23" s="37">
-        <f>Métricas!E24</f>
+        <f>Métricas!E25</f>
         <v>3.450655624568668E-3</v>
       </c>
       <c r="J23" s="9" t="str">
@@ -7478,7 +7534,7 @@
         <v/>
       </c>
       <c r="Q23" s="10" t="str">
-        <f>IFERROR("Ganhos na alienação de ativos — 2023: "&amp;ROUND(Métricas!C23,0)&amp;"; 2024: "&amp;ROUND(Métricas!D23,0)&amp;"; 2025: "&amp;ROUND(Métricas!E23,0)&amp;" ("&amp;ROUND(Métricas!E24*100,1)&amp;"%"&amp;" do EBITDA). EBITDA de 2025 sem esses ganhos: "&amp;ROUND(Métricas!E25,0)&amp;". Fonte: "&amp;Input!$F$44&amp;"; "&amp;Input!$F$11,"Ver folha Métricas")</f>
+        <f>IFERROR("Ganhos na alienação de ativos — 2023: "&amp;ROUND(Métricas!C24,0)&amp;"; 2024: "&amp;ROUND(Métricas!D24,0)&amp;"; 2025: "&amp;ROUND(Métricas!E24,0)&amp;" ("&amp;ROUND(Métricas!E25*100,1)&amp;"%"&amp;" do EBITDA). EBITDA de 2025 sem esses ganhos: "&amp;ROUND(Métricas!E26,0)&amp;". Fonte: "&amp;Input!$F$44&amp;"; "&amp;Input!$F$11,"Ver folha Métricas")</f>
         <v>Ganhos na alienação de ativos — 2023: 0; 2024: 0; 2025: 5 (0,3% do EBITDA). EBITDA de 2025 sem esses ganhos: 1444. Fonte: DFC!B9:D9; DRE!B11:D11</v>
       </c>
       <c r="R23" s="10" t="s">
@@ -7498,7 +7554,7 @@
         <v>R19 · Ganho na venda de ativos dentro do EBITDA (limite: 5%)</v>
       </c>
     </row>
-    <row r="24" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:22" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
         <v>426</v>
       </c>
@@ -7518,15 +7574,15 @@
         <v>0.15</v>
       </c>
       <c r="G24" s="37" t="str">
-        <f>Métricas!C55</f>
+        <f>Métricas!C57</f>
         <v>n.d.</v>
       </c>
       <c r="H24" s="37" t="str">
-        <f>Métricas!D55</f>
+        <f>Métricas!D57</f>
         <v>n.d.</v>
       </c>
       <c r="I24" s="37">
-        <f>Métricas!E55</f>
+        <f>Métricas!E57</f>
         <v>0.82355647573038882</v>
       </c>
       <c r="J24" s="9" t="str">
@@ -7557,7 +7613,7 @@
         <v/>
       </c>
       <c r="Q24" s="10" t="str">
-        <f>IFERROR("Dívida líquida / EBITDA em 2025: "&amp;ROUND(Métricas!E52,2)&amp;"x (limite "&amp;ROUND(Métricas!E54,1)&amp;"x); folga de "&amp;ROUND(Métricas!E55*100,1)&amp;"%"&amp;". EBITDA mínimo para cumprir: "&amp;ROUND(Métricas!E56,0)&amp;". Sem ganhos na alienação, o rácio é "&amp;ROUND(Métricas!E53,2)&amp;"x. Fonte: "&amp;Input!$F$73&amp;"; "&amp;Input!$F$30,"Ver folha Métricas")</f>
+        <f>IFERROR("Dívida líquida / EBITDA em 2025: "&amp;ROUND(Métricas!E54,2)&amp;"x (limite "&amp;ROUND(Métricas!E56,1)&amp;"x); folga de "&amp;ROUND(Métricas!E57*100,1)&amp;"%"&amp;". EBITDA mínimo para cumprir: "&amp;ROUND(Métricas!E58,0)&amp;". Sem ganhos na alienação, o rácio é "&amp;ROUND(Métricas!E55,2)&amp;"x. Fonte: "&amp;Input!$F$73&amp;"; "&amp;Input!$F$30,"Ver folha Métricas")</f>
         <v>Dívida líquida / EBITDA em 2025: 0,53x (limite 3x); folga de 82,4%. EBITDA mínimo para cumprir: 256. Sem ganhos na alienação, o rácio é 0,53x. Fonte: Dívida!I5 (empréstimo bancário, teste anual); Balanço!B23:E23</v>
       </c>
       <c r="R24" s="10" t="s">

</xml_diff>